<commit_message>
Add EMPTY Projection.Mode for unconstrained params and fix activity limits
- Add set_empty_projection_mode_for_investment_params() to mark investment
  parameters as EMPTY so B1_Compiler omits them (unconstrained in OSeMOSYS)
- Fix activity limits: write None instead of 0 for empty years, set
  Projection.Mode to EMPTY when all years are empty
- Simplify upper limit formula to LowerLimit × 1.05 (remove fixed +0.1 margin)
- Fix demand adjustments to read from olade_config instead of ostram_config
- Only skip manual ResidualCapacity for techs that OLADE actually covers
- Add auxiliary scripts for RES diagrams and transmission maps
- Add centerpoints.csv and update output files for all scenarios
</commit_message>
<xml_diff>
--- a/t1_confection/A1_Outputs/A1_Outputs_BAU/A-O_Demand.xlsx
+++ b/t1_confection/A1_Outputs/A1_Outputs_BAU/A-O_Demand.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ19"/>
+  <dimension ref="A1:AJ20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.85546875" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
@@ -750,88 +750,88 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>611.17</v>
+        <v>524.49</v>
       </c>
       <c r="J2" t="n">
-        <v>588.9400000000001</v>
+        <v>506.39</v>
       </c>
       <c r="K2" t="n">
-        <v>588.03</v>
+        <v>509.61</v>
       </c>
       <c r="L2" t="n">
-        <v>600.02</v>
+        <v>513.74</v>
       </c>
       <c r="M2" t="n">
-        <v>612</v>
+        <v>517.87</v>
       </c>
       <c r="N2" t="n">
-        <v>623.99</v>
+        <v>522</v>
       </c>
       <c r="O2" t="n">
-        <v>635.97</v>
+        <v>526.13</v>
       </c>
       <c r="P2" t="n">
-        <v>647.95</v>
+        <v>530.25</v>
       </c>
       <c r="Q2" t="n">
-        <v>662.34</v>
+        <v>534.38</v>
       </c>
       <c r="R2" t="n">
-        <v>676.73</v>
+        <v>538.51</v>
       </c>
       <c r="S2" t="n">
-        <v>691.12</v>
+        <v>542.64</v>
       </c>
       <c r="T2" t="n">
-        <v>705.5</v>
+        <v>546.77</v>
       </c>
       <c r="U2" t="n">
-        <v>719.89</v>
+        <v>550.9</v>
       </c>
       <c r="V2" t="n">
-        <v>735.12</v>
+        <v>555.03</v>
       </c>
       <c r="W2" t="n">
-        <v>750.35</v>
+        <v>559.16</v>
       </c>
       <c r="X2" t="n">
-        <v>765.58</v>
+        <v>563.29</v>
       </c>
       <c r="Y2" t="n">
-        <v>780.8200000000001</v>
+        <v>567.42</v>
       </c>
       <c r="Z2" t="n">
-        <v>796.05</v>
+        <v>571.55</v>
       </c>
       <c r="AA2" t="n">
-        <v>810.9299999999999</v>
+        <v>575.6799999999999</v>
       </c>
       <c r="AB2" t="n">
-        <v>825.8099999999999</v>
+        <v>579.8099999999999</v>
       </c>
       <c r="AC2" t="n">
-        <v>840.7</v>
+        <v>583.9299999999999</v>
       </c>
       <c r="AD2" t="n">
-        <v>855.58</v>
+        <v>588.0599999999999</v>
       </c>
       <c r="AE2" t="n">
-        <v>870.46</v>
+        <v>592.1900000000001</v>
       </c>
       <c r="AF2" t="n">
-        <v>885.64</v>
+        <v>596.3200000000001</v>
       </c>
       <c r="AG2" t="n">
-        <v>900.8200000000001</v>
+        <v>600.45</v>
       </c>
       <c r="AH2" t="n">
-        <v>916</v>
+        <v>604.58</v>
       </c>
       <c r="AI2" t="n">
-        <v>931.1799999999999</v>
+        <v>608.71</v>
       </c>
       <c r="AJ2" t="n">
-        <v>946.35</v>
+        <v>612.84</v>
       </c>
     </row>
     <row r="3">
@@ -874,88 +874,88 @@
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>48.22</v>
+        <v>42.81</v>
       </c>
       <c r="J3" t="n">
-        <v>49.89</v>
+        <v>45.15</v>
       </c>
       <c r="K3" t="n">
-        <v>52.46</v>
+        <v>48.39</v>
       </c>
       <c r="L3" t="n">
-        <v>54.88</v>
+        <v>51.14</v>
       </c>
       <c r="M3" t="n">
-        <v>57.3</v>
+        <v>53.88</v>
       </c>
       <c r="N3" t="n">
-        <v>59.73</v>
+        <v>56.63</v>
       </c>
       <c r="O3" t="n">
-        <v>62.15</v>
+        <v>59.38</v>
       </c>
       <c r="P3" t="n">
-        <v>64.56999999999999</v>
+        <v>62.13</v>
       </c>
       <c r="Q3" t="n">
-        <v>67.27</v>
+        <v>64.88</v>
       </c>
       <c r="R3" t="n">
-        <v>69.97</v>
+        <v>67.63</v>
       </c>
       <c r="S3" t="n">
-        <v>72.66</v>
+        <v>70.37</v>
       </c>
       <c r="T3" t="n">
-        <v>75.36</v>
+        <v>73.12</v>
       </c>
       <c r="U3" t="n">
-        <v>78.06</v>
+        <v>75.87</v>
       </c>
       <c r="V3" t="n">
-        <v>81.15000000000001</v>
+        <v>78.62</v>
       </c>
       <c r="W3" t="n">
-        <v>84.23999999999999</v>
+        <v>81.37</v>
       </c>
       <c r="X3" t="n">
-        <v>87.33</v>
+        <v>84.12</v>
       </c>
       <c r="Y3" t="n">
-        <v>90.42</v>
+        <v>86.87</v>
       </c>
       <c r="Z3" t="n">
-        <v>93.51000000000001</v>
+        <v>89.61</v>
       </c>
       <c r="AA3" t="n">
-        <v>97.04000000000001</v>
+        <v>92.36</v>
       </c>
       <c r="AB3" t="n">
-        <v>100.57</v>
+        <v>95.11</v>
       </c>
       <c r="AC3" t="n">
-        <v>104.1</v>
+        <v>97.86</v>
       </c>
       <c r="AD3" t="n">
-        <v>107.63</v>
+        <v>100.61</v>
       </c>
       <c r="AE3" t="n">
-        <v>111.16</v>
+        <v>103.36</v>
       </c>
       <c r="AF3" t="n">
-        <v>115.22</v>
+        <v>106.1</v>
       </c>
       <c r="AG3" t="n">
-        <v>119.27</v>
+        <v>108.85</v>
       </c>
       <c r="AH3" t="n">
-        <v>123.33</v>
+        <v>111.6</v>
       </c>
       <c r="AI3" t="n">
-        <v>127.39</v>
+        <v>114.35</v>
       </c>
       <c r="AJ3" t="n">
-        <v>131.44</v>
+        <v>117.1</v>
       </c>
     </row>
     <row r="4">
@@ -998,88 +998,88 @@
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>2268.28</v>
+        <v>2599.63</v>
       </c>
       <c r="J4" t="n">
-        <v>2250.4</v>
+        <v>2637.58</v>
       </c>
       <c r="K4" t="n">
-        <v>2276.48</v>
+        <v>2719.49</v>
       </c>
       <c r="L4" t="n">
-        <v>2276.48</v>
+        <v>2775.31</v>
       </c>
       <c r="M4" t="n">
-        <v>2276.48</v>
+        <v>2831.14</v>
       </c>
       <c r="N4" t="n">
-        <v>2276.48</v>
+        <v>2886.97</v>
       </c>
       <c r="O4" t="n">
-        <v>2276.48</v>
+        <v>2942.8</v>
       </c>
       <c r="P4" t="n">
-        <v>2276.48</v>
+        <v>2998.63</v>
       </c>
       <c r="Q4" t="n">
-        <v>2297.99</v>
+        <v>3054.45</v>
       </c>
       <c r="R4" t="n">
-        <v>2319.51</v>
+        <v>3110.28</v>
       </c>
       <c r="S4" t="n">
-        <v>2341.05</v>
+        <v>3166.11</v>
       </c>
       <c r="T4" t="n">
-        <v>2362.56</v>
+        <v>3221.94</v>
       </c>
       <c r="U4" t="n">
-        <v>2384.08</v>
+        <v>3277.77</v>
       </c>
       <c r="V4" t="n">
-        <v>2424.3</v>
+        <v>3333.59</v>
       </c>
       <c r="W4" t="n">
-        <v>2464.55</v>
+        <v>3389.42</v>
       </c>
       <c r="X4" t="n">
-        <v>2504.79</v>
+        <v>3445.25</v>
       </c>
       <c r="Y4" t="n">
-        <v>2545.03</v>
+        <v>3501.08</v>
       </c>
       <c r="Z4" t="n">
-        <v>2585.28</v>
+        <v>3556.91</v>
       </c>
       <c r="AA4" t="n">
-        <v>2624.3</v>
+        <v>3612.74</v>
       </c>
       <c r="AB4" t="n">
-        <v>2663.31</v>
+        <v>3668.56</v>
       </c>
       <c r="AC4" t="n">
-        <v>2702.33</v>
+        <v>3724.39</v>
       </c>
       <c r="AD4" t="n">
-        <v>2741.33</v>
+        <v>3780.22</v>
       </c>
       <c r="AE4" t="n">
-        <v>2780.36</v>
+        <v>3836.05</v>
       </c>
       <c r="AF4" t="n">
-        <v>2819.64</v>
+        <v>3891.88</v>
       </c>
       <c r="AG4" t="n">
-        <v>2858.91</v>
+        <v>3947.7</v>
       </c>
       <c r="AH4" t="n">
-        <v>2898.19</v>
+        <v>4003.53</v>
       </c>
       <c r="AI4" t="n">
-        <v>2937.47</v>
+        <v>4059.36</v>
       </c>
       <c r="AJ4" t="n">
-        <v>2976.75</v>
+        <v>4115.19</v>
       </c>
     </row>
     <row r="5">
@@ -1122,88 +1122,88 @@
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>14.87</v>
+        <v>3.87</v>
       </c>
       <c r="J5" t="n">
-        <v>14.87</v>
+        <v>4.12</v>
       </c>
       <c r="K5" t="n">
-        <v>14.87</v>
+        <v>4.37</v>
       </c>
       <c r="L5" t="n">
-        <v>14.87</v>
+        <v>4.62</v>
       </c>
       <c r="M5" t="n">
-        <v>14.87</v>
+        <v>4.86</v>
       </c>
       <c r="N5" t="n">
-        <v>14.87</v>
+        <v>5.11</v>
       </c>
       <c r="O5" t="n">
-        <v>14.87</v>
+        <v>5.36</v>
       </c>
       <c r="P5" t="n">
-        <v>14.87</v>
+        <v>5.6</v>
       </c>
       <c r="Q5" t="n">
-        <v>14.87</v>
+        <v>5.85</v>
       </c>
       <c r="R5" t="n">
-        <v>14.87</v>
+        <v>6.1</v>
       </c>
       <c r="S5" t="n">
-        <v>14.87</v>
+        <v>6.35</v>
       </c>
       <c r="T5" t="n">
-        <v>14.87</v>
+        <v>6.59</v>
       </c>
       <c r="U5" t="n">
-        <v>14.87</v>
+        <v>6.84</v>
       </c>
       <c r="V5" t="n">
-        <v>14.87</v>
+        <v>7.09</v>
       </c>
       <c r="W5" t="n">
-        <v>14.87</v>
+        <v>7.33</v>
       </c>
       <c r="X5" t="n">
-        <v>14.87</v>
+        <v>7.58</v>
       </c>
       <c r="Y5" t="n">
-        <v>14.87</v>
+        <v>7.83</v>
       </c>
       <c r="Z5" t="n">
-        <v>14.87</v>
+        <v>8.08</v>
       </c>
       <c r="AA5" t="n">
-        <v>14.88</v>
+        <v>8.32</v>
       </c>
       <c r="AB5" t="n">
-        <v>14.88</v>
+        <v>8.57</v>
       </c>
       <c r="AC5" t="n">
-        <v>14.89</v>
+        <v>8.82</v>
       </c>
       <c r="AD5" t="n">
-        <v>14.9</v>
+        <v>9.06</v>
       </c>
       <c r="AE5" t="n">
-        <v>14.9</v>
+        <v>9.31</v>
       </c>
       <c r="AF5" t="n">
-        <v>15.73</v>
+        <v>9.56</v>
       </c>
       <c r="AG5" t="n">
-        <v>16.55</v>
+        <v>9.81</v>
       </c>
       <c r="AH5" t="n">
-        <v>17.37</v>
+        <v>10.05</v>
       </c>
       <c r="AI5" t="n">
-        <v>18.19</v>
+        <v>10.3</v>
       </c>
       <c r="AJ5" t="n">
-        <v>19.02</v>
+        <v>10.55</v>
       </c>
     </row>
     <row r="6">
@@ -1246,88 +1246,88 @@
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>271.26</v>
+        <v>302.25</v>
       </c>
       <c r="J6" t="n">
-        <v>271.4</v>
+        <v>318.54</v>
       </c>
       <c r="K6" t="n">
-        <v>271.37</v>
+        <v>334.66</v>
       </c>
       <c r="L6" t="n">
-        <v>271.37</v>
+        <v>350.81</v>
       </c>
       <c r="M6" t="n">
-        <v>271.37</v>
+        <v>366.95</v>
       </c>
       <c r="N6" t="n">
-        <v>271.37</v>
+        <v>383.1</v>
       </c>
       <c r="O6" t="n">
-        <v>271.37</v>
+        <v>399.25</v>
       </c>
       <c r="P6" t="n">
-        <v>271.37</v>
+        <v>415.4</v>
       </c>
       <c r="Q6" t="n">
-        <v>272.87</v>
+        <v>431.54</v>
       </c>
       <c r="R6" t="n">
-        <v>274.37</v>
+        <v>447.69</v>
       </c>
       <c r="S6" t="n">
-        <v>275.86</v>
+        <v>463.84</v>
       </c>
       <c r="T6" t="n">
-        <v>277.36</v>
+        <v>479.99</v>
       </c>
       <c r="U6" t="n">
-        <v>278.85</v>
+        <v>496.14</v>
       </c>
       <c r="V6" t="n">
-        <v>284.91</v>
+        <v>512.28</v>
       </c>
       <c r="W6" t="n">
-        <v>290.97</v>
+        <v>528.4299999999999</v>
       </c>
       <c r="X6" t="n">
-        <v>297.03</v>
+        <v>544.58</v>
       </c>
       <c r="Y6" t="n">
-        <v>303.09</v>
+        <v>560.73</v>
       </c>
       <c r="Z6" t="n">
-        <v>309.16</v>
+        <v>576.87</v>
       </c>
       <c r="AA6" t="n">
-        <v>315.46</v>
+        <v>593.02</v>
       </c>
       <c r="AB6" t="n">
-        <v>321.76</v>
+        <v>609.17</v>
       </c>
       <c r="AC6" t="n">
-        <v>328.07</v>
+        <v>625.3200000000001</v>
       </c>
       <c r="AD6" t="n">
-        <v>334.37</v>
+        <v>641.47</v>
       </c>
       <c r="AE6" t="n">
-        <v>340.68</v>
+        <v>657.61</v>
       </c>
       <c r="AF6" t="n">
-        <v>346.97</v>
+        <v>673.76</v>
       </c>
       <c r="AG6" t="n">
-        <v>353.26</v>
+        <v>689.91</v>
       </c>
       <c r="AH6" t="n">
-        <v>359.55</v>
+        <v>706.0599999999999</v>
       </c>
       <c r="AI6" t="n">
-        <v>365.84</v>
+        <v>722.2</v>
       </c>
       <c r="AJ6" t="n">
-        <v>372.13</v>
+        <v>738.35</v>
       </c>
     </row>
     <row r="7">
@@ -1370,88 +1370,88 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>381.42</v>
+        <v>288.23</v>
       </c>
       <c r="J7" t="n">
-        <v>388.96</v>
+        <v>296.14</v>
       </c>
       <c r="K7" t="n">
-        <v>403.26</v>
+        <v>310.83</v>
       </c>
       <c r="L7" t="n">
-        <v>415.05</v>
+        <v>321.53</v>
       </c>
       <c r="M7" t="n">
-        <v>426.83</v>
+        <v>332.24</v>
       </c>
       <c r="N7" t="n">
-        <v>438.62</v>
+        <v>342.94</v>
       </c>
       <c r="O7" t="n">
-        <v>450.41</v>
+        <v>353.65</v>
       </c>
       <c r="P7" t="n">
-        <v>462.19</v>
+        <v>364.35</v>
       </c>
       <c r="Q7" t="n">
-        <v>475.02</v>
+        <v>375.05</v>
       </c>
       <c r="R7" t="n">
-        <v>487.85</v>
+        <v>385.76</v>
       </c>
       <c r="S7" t="n">
-        <v>500.68</v>
+        <v>396.46</v>
       </c>
       <c r="T7" t="n">
-        <v>513.5</v>
+        <v>407.17</v>
       </c>
       <c r="U7" t="n">
-        <v>526.33</v>
+        <v>417.87</v>
       </c>
       <c r="V7" t="n">
-        <v>540.62</v>
+        <v>428.58</v>
       </c>
       <c r="W7" t="n">
-        <v>554.91</v>
+        <v>439.28</v>
       </c>
       <c r="X7" t="n">
-        <v>569.1900000000001</v>
+        <v>449.98</v>
       </c>
       <c r="Y7" t="n">
-        <v>583.48</v>
+        <v>460.69</v>
       </c>
       <c r="Z7" t="n">
-        <v>597.77</v>
+        <v>471.39</v>
       </c>
       <c r="AA7" t="n">
-        <v>613.33</v>
+        <v>482.1</v>
       </c>
       <c r="AB7" t="n">
-        <v>628.89</v>
+        <v>492.8</v>
       </c>
       <c r="AC7" t="n">
-        <v>644.46</v>
+        <v>503.51</v>
       </c>
       <c r="AD7" t="n">
-        <v>660.02</v>
+        <v>514.21</v>
       </c>
       <c r="AE7" t="n">
-        <v>675.59</v>
+        <v>524.91</v>
       </c>
       <c r="AF7" t="n">
-        <v>692.27</v>
+        <v>535.62</v>
       </c>
       <c r="AG7" t="n">
-        <v>708.96</v>
+        <v>546.3200000000001</v>
       </c>
       <c r="AH7" t="n">
-        <v>725.64</v>
+        <v>557.03</v>
       </c>
       <c r="AI7" t="n">
-        <v>742.33</v>
+        <v>567.73</v>
       </c>
       <c r="AJ7" t="n">
-        <v>759.01</v>
+        <v>578.4400000000001</v>
       </c>
     </row>
     <row r="8">
@@ -1494,88 +1494,88 @@
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>46.71</v>
+        <v>44.28</v>
       </c>
       <c r="J8" t="n">
-        <v>48.51</v>
+        <v>44.68</v>
       </c>
       <c r="K8" t="n">
-        <v>48.82</v>
+        <v>43.57</v>
       </c>
       <c r="L8" t="n">
-        <v>51.52</v>
+        <v>44.46</v>
       </c>
       <c r="M8" t="n">
-        <v>54.23</v>
+        <v>45.34</v>
       </c>
       <c r="N8" t="n">
-        <v>56.93</v>
+        <v>46.23</v>
       </c>
       <c r="O8" t="n">
-        <v>59.64</v>
+        <v>47.12</v>
       </c>
       <c r="P8" t="n">
-        <v>62.35</v>
+        <v>48</v>
       </c>
       <c r="Q8" t="n">
-        <v>65.31</v>
+        <v>48.89</v>
       </c>
       <c r="R8" t="n">
-        <v>68.27</v>
+        <v>49.77</v>
       </c>
       <c r="S8" t="n">
-        <v>71.23</v>
+        <v>50.66</v>
       </c>
       <c r="T8" t="n">
-        <v>74.19</v>
+        <v>51.54</v>
       </c>
       <c r="U8" t="n">
-        <v>77.15000000000001</v>
+        <v>52.43</v>
       </c>
       <c r="V8" t="n">
-        <v>80.5</v>
+        <v>53.31</v>
       </c>
       <c r="W8" t="n">
-        <v>83.84999999999999</v>
+        <v>54.2</v>
       </c>
       <c r="X8" t="n">
-        <v>87.19</v>
+        <v>55.08</v>
       </c>
       <c r="Y8" t="n">
-        <v>90.54000000000001</v>
+        <v>55.97</v>
       </c>
       <c r="Z8" t="n">
-        <v>93.89</v>
+        <v>56.86</v>
       </c>
       <c r="AA8" t="n">
-        <v>97.53</v>
+        <v>57.74</v>
       </c>
       <c r="AB8" t="n">
-        <v>101.18</v>
+        <v>58.63</v>
       </c>
       <c r="AC8" t="n">
-        <v>104.82</v>
+        <v>59.51</v>
       </c>
       <c r="AD8" t="n">
-        <v>108.46</v>
+        <v>60.4</v>
       </c>
       <c r="AE8" t="n">
-        <v>112.11</v>
+        <v>61.28</v>
       </c>
       <c r="AF8" t="n">
-        <v>115.95</v>
+        <v>62.17</v>
       </c>
       <c r="AG8" t="n">
-        <v>119.78</v>
+        <v>63.05</v>
       </c>
       <c r="AH8" t="n">
-        <v>123.62</v>
+        <v>63.94</v>
       </c>
       <c r="AI8" t="n">
-        <v>127.46</v>
+        <v>64.81999999999999</v>
       </c>
       <c r="AJ8" t="n">
-        <v>131.29</v>
+        <v>65.70999999999999</v>
       </c>
     </row>
     <row r="9">
@@ -1618,88 +1618,88 @@
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>66.8</v>
+        <v>86.09</v>
       </c>
       <c r="J9" t="n">
-        <v>66.92</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="K9" t="n">
-        <v>67.03</v>
+        <v>92.11</v>
       </c>
       <c r="L9" t="n">
-        <v>71.7</v>
+        <v>95.12</v>
       </c>
       <c r="M9" t="n">
-        <v>76.37</v>
+        <v>98.14</v>
       </c>
       <c r="N9" t="n">
-        <v>81.04000000000001</v>
+        <v>101.15</v>
       </c>
       <c r="O9" t="n">
-        <v>85.7</v>
+        <v>104.16</v>
       </c>
       <c r="P9" t="n">
-        <v>90.37</v>
+        <v>107.18</v>
       </c>
       <c r="Q9" t="n">
-        <v>95.44</v>
+        <v>110.19</v>
       </c>
       <c r="R9" t="n">
-        <v>100.51</v>
+        <v>113.2</v>
       </c>
       <c r="S9" t="n">
-        <v>105.58</v>
+        <v>116.21</v>
       </c>
       <c r="T9" t="n">
-        <v>110.65</v>
+        <v>119.23</v>
       </c>
       <c r="U9" t="n">
-        <v>115.72</v>
+        <v>122.24</v>
       </c>
       <c r="V9" t="n">
-        <v>121.48</v>
+        <v>125.25</v>
       </c>
       <c r="W9" t="n">
-        <v>127.23</v>
+        <v>128.27</v>
       </c>
       <c r="X9" t="n">
-        <v>132.98</v>
+        <v>131.28</v>
       </c>
       <c r="Y9" t="n">
-        <v>138.73</v>
+        <v>134.29</v>
       </c>
       <c r="Z9" t="n">
-        <v>144.49</v>
+        <v>137.31</v>
       </c>
       <c r="AA9" t="n">
-        <v>150.83</v>
+        <v>140.32</v>
       </c>
       <c r="AB9" t="n">
-        <v>157.18</v>
+        <v>143.33</v>
       </c>
       <c r="AC9" t="n">
-        <v>163.53</v>
+        <v>146.34</v>
       </c>
       <c r="AD9" t="n">
-        <v>169.88</v>
+        <v>149.36</v>
       </c>
       <c r="AE9" t="n">
-        <v>176.23</v>
+        <v>152.37</v>
       </c>
       <c r="AF9" t="n">
-        <v>183.07</v>
+        <v>155.38</v>
       </c>
       <c r="AG9" t="n">
-        <v>189.91</v>
+        <v>158.4</v>
       </c>
       <c r="AH9" t="n">
-        <v>196.75</v>
+        <v>161.41</v>
       </c>
       <c r="AI9" t="n">
-        <v>203.59</v>
+        <v>164.42</v>
       </c>
       <c r="AJ9" t="n">
-        <v>210.44</v>
+        <v>167.44</v>
       </c>
     </row>
     <row r="10">
@@ -1742,88 +1742,88 @@
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>99.68000000000001</v>
+        <v>129.57</v>
       </c>
       <c r="J10" t="n">
-        <v>102.97</v>
+        <v>137.75</v>
       </c>
       <c r="K10" t="n">
-        <v>99.95</v>
+        <v>139.6</v>
       </c>
       <c r="L10" t="n">
-        <v>103.13</v>
+        <v>145.41</v>
       </c>
       <c r="M10" t="n">
-        <v>106.32</v>
+        <v>151.21</v>
       </c>
       <c r="N10" t="n">
-        <v>109.5</v>
+        <v>157.02</v>
       </c>
       <c r="O10" t="n">
-        <v>112.68</v>
+        <v>162.82</v>
       </c>
       <c r="P10" t="n">
-        <v>115.87</v>
+        <v>168.63</v>
       </c>
       <c r="Q10" t="n">
-        <v>119.33</v>
+        <v>174.43</v>
       </c>
       <c r="R10" t="n">
-        <v>122.8</v>
+        <v>180.24</v>
       </c>
       <c r="S10" t="n">
-        <v>126.27</v>
+        <v>186.04</v>
       </c>
       <c r="T10" t="n">
-        <v>129.73</v>
+        <v>191.85</v>
       </c>
       <c r="U10" t="n">
-        <v>133.2</v>
+        <v>197.65</v>
       </c>
       <c r="V10" t="n">
-        <v>137.2</v>
+        <v>203.46</v>
       </c>
       <c r="W10" t="n">
-        <v>141.2</v>
+        <v>209.26</v>
       </c>
       <c r="X10" t="n">
-        <v>145.2</v>
+        <v>215.07</v>
       </c>
       <c r="Y10" t="n">
-        <v>149.21</v>
+        <v>220.87</v>
       </c>
       <c r="Z10" t="n">
-        <v>153.21</v>
+        <v>226.68</v>
       </c>
       <c r="AA10" t="n">
-        <v>157.85</v>
+        <v>232.48</v>
       </c>
       <c r="AB10" t="n">
-        <v>162.5</v>
+        <v>238.29</v>
       </c>
       <c r="AC10" t="n">
-        <v>167.15</v>
+        <v>244.09</v>
       </c>
       <c r="AD10" t="n">
-        <v>171.79</v>
+        <v>249.9</v>
       </c>
       <c r="AE10" t="n">
-        <v>176.44</v>
+        <v>255.7</v>
       </c>
       <c r="AF10" t="n">
-        <v>181.73</v>
+        <v>261.51</v>
       </c>
       <c r="AG10" t="n">
-        <v>187.02</v>
+        <v>267.31</v>
       </c>
       <c r="AH10" t="n">
-        <v>192.3</v>
+        <v>273.12</v>
       </c>
       <c r="AI10" t="n">
-        <v>197.59</v>
+        <v>278.92</v>
       </c>
       <c r="AJ10" t="n">
-        <v>202.88</v>
+        <v>284.73</v>
       </c>
     </row>
     <row r="11">
@@ -1866,88 +1866,88 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>41.19</v>
+        <v>47.17</v>
       </c>
       <c r="J11" t="n">
-        <v>41.03</v>
+        <v>48.54</v>
       </c>
       <c r="K11" t="n">
-        <v>39.49</v>
+        <v>48.53</v>
       </c>
       <c r="L11" t="n">
-        <v>39.49</v>
+        <v>50.07</v>
       </c>
       <c r="M11" t="n">
-        <v>39.49</v>
+        <v>51.6</v>
       </c>
       <c r="N11" t="n">
-        <v>39.49</v>
+        <v>53.13</v>
       </c>
       <c r="O11" t="n">
-        <v>39.49</v>
+        <v>54.66</v>
       </c>
       <c r="P11" t="n">
-        <v>39.49</v>
+        <v>56.19</v>
       </c>
       <c r="Q11" t="n">
-        <v>39.49</v>
+        <v>57.72</v>
       </c>
       <c r="R11" t="n">
-        <v>39.49</v>
+        <v>59.25</v>
       </c>
       <c r="S11" t="n">
-        <v>39.49</v>
+        <v>60.79</v>
       </c>
       <c r="T11" t="n">
-        <v>39.49</v>
+        <v>62.32</v>
       </c>
       <c r="U11" t="n">
-        <v>39.49</v>
+        <v>63.85</v>
       </c>
       <c r="V11" t="n">
-        <v>42.01</v>
+        <v>65.38</v>
       </c>
       <c r="W11" t="n">
-        <v>44.53</v>
+        <v>66.91</v>
       </c>
       <c r="X11" t="n">
-        <v>47.05</v>
+        <v>68.44</v>
       </c>
       <c r="Y11" t="n">
-        <v>49.56</v>
+        <v>69.97</v>
       </c>
       <c r="Z11" t="n">
-        <v>52.08</v>
+        <v>71.5</v>
       </c>
       <c r="AA11" t="n">
-        <v>60.47</v>
+        <v>73.04000000000001</v>
       </c>
       <c r="AB11" t="n">
-        <v>68.84999999999999</v>
+        <v>74.56999999999999</v>
       </c>
       <c r="AC11" t="n">
-        <v>77.23999999999999</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="AD11" t="n">
-        <v>85.62</v>
+        <v>77.63</v>
       </c>
       <c r="AE11" t="n">
-        <v>94.01000000000001</v>
+        <v>79.16</v>
       </c>
       <c r="AF11" t="n">
-        <v>104.66</v>
+        <v>80.69</v>
       </c>
       <c r="AG11" t="n">
-        <v>115.32</v>
+        <v>82.22</v>
       </c>
       <c r="AH11" t="n">
-        <v>125.98</v>
+        <v>83.75</v>
       </c>
       <c r="AI11" t="n">
-        <v>136.63</v>
+        <v>85.29000000000001</v>
       </c>
       <c r="AJ11" t="n">
-        <v>147.29</v>
+        <v>86.81999999999999</v>
       </c>
     </row>
     <row r="12">
@@ -1990,88 +1990,88 @@
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>33.3</v>
+        <v>43.14</v>
       </c>
       <c r="J12" t="n">
-        <v>33.32</v>
+        <v>44.46</v>
       </c>
       <c r="K12" t="n">
-        <v>33.49</v>
+        <v>45.94</v>
       </c>
       <c r="L12" t="n">
-        <v>33.49</v>
+        <v>47.24</v>
       </c>
       <c r="M12" t="n">
-        <v>33.49</v>
+        <v>48.55</v>
       </c>
       <c r="N12" t="n">
-        <v>33.49</v>
+        <v>49.85</v>
       </c>
       <c r="O12" t="n">
-        <v>33.49</v>
+        <v>51.16</v>
       </c>
       <c r="P12" t="n">
-        <v>33.49</v>
+        <v>52.46</v>
       </c>
       <c r="Q12" t="n">
-        <v>33.49</v>
+        <v>53.77</v>
       </c>
       <c r="R12" t="n">
-        <v>33.49</v>
+        <v>55.07</v>
       </c>
       <c r="S12" t="n">
-        <v>33.49</v>
+        <v>56.38</v>
       </c>
       <c r="T12" t="n">
-        <v>33.49</v>
+        <v>57.68</v>
       </c>
       <c r="U12" t="n">
-        <v>33.49</v>
+        <v>58.98</v>
       </c>
       <c r="V12" t="n">
-        <v>33.49</v>
+        <v>60.29</v>
       </c>
       <c r="W12" t="n">
-        <v>33.49</v>
+        <v>61.59</v>
       </c>
       <c r="X12" t="n">
-        <v>33.49</v>
+        <v>62.9</v>
       </c>
       <c r="Y12" t="n">
-        <v>33.49</v>
+        <v>64.2</v>
       </c>
       <c r="Z12" t="n">
-        <v>33.49</v>
+        <v>65.51000000000001</v>
       </c>
       <c r="AA12" t="n">
-        <v>33.49</v>
+        <v>66.81</v>
       </c>
       <c r="AB12" t="n">
-        <v>33.49</v>
+        <v>68.12</v>
       </c>
       <c r="AC12" t="n">
-        <v>33.49</v>
+        <v>69.42</v>
       </c>
       <c r="AD12" t="n">
-        <v>33.49</v>
+        <v>70.73</v>
       </c>
       <c r="AE12" t="n">
-        <v>33.49</v>
+        <v>72.03</v>
       </c>
       <c r="AF12" t="n">
-        <v>38.18</v>
+        <v>73.34</v>
       </c>
       <c r="AG12" t="n">
-        <v>42.88</v>
+        <v>74.64</v>
       </c>
       <c r="AH12" t="n">
-        <v>47.58</v>
+        <v>75.95</v>
       </c>
       <c r="AI12" t="n">
-        <v>52.28</v>
+        <v>77.25</v>
       </c>
       <c r="AJ12" t="n">
-        <v>56.97</v>
+        <v>78.56</v>
       </c>
     </row>
     <row r="13">
@@ -2114,88 +2114,88 @@
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>1206.65</v>
+        <v>1241.42</v>
       </c>
       <c r="J13" t="n">
-        <v>1238.93</v>
+        <v>1279.49</v>
       </c>
       <c r="K13" t="n">
-        <v>1271.38</v>
+        <v>1317.71</v>
       </c>
       <c r="L13" t="n">
-        <v>1335.71</v>
+        <v>1355.13</v>
       </c>
       <c r="M13" t="n">
-        <v>1400.04</v>
+        <v>1392.55</v>
       </c>
       <c r="N13" t="n">
-        <v>1464.38</v>
+        <v>1429.98</v>
       </c>
       <c r="O13" t="n">
-        <v>1528.71</v>
+        <v>1467.4</v>
       </c>
       <c r="P13" t="n">
-        <v>1593.04</v>
+        <v>1504.82</v>
       </c>
       <c r="Q13" t="n">
-        <v>1663.64</v>
+        <v>1542.24</v>
       </c>
       <c r="R13" t="n">
-        <v>1734.23</v>
+        <v>1579.67</v>
       </c>
       <c r="S13" t="n">
-        <v>1804.83</v>
+        <v>1617.09</v>
       </c>
       <c r="T13" t="n">
-        <v>1875.42</v>
+        <v>1654.51</v>
       </c>
       <c r="U13" t="n">
-        <v>1946.02</v>
+        <v>1691.93</v>
       </c>
       <c r="V13" t="n">
-        <v>2022.61</v>
+        <v>1729.36</v>
       </c>
       <c r="W13" t="n">
-        <v>2099.2</v>
+        <v>1766.78</v>
       </c>
       <c r="X13" t="n">
-        <v>2175.79</v>
+        <v>1804.2</v>
       </c>
       <c r="Y13" t="n">
-        <v>2252.39</v>
+        <v>1841.62</v>
       </c>
       <c r="Z13" t="n">
-        <v>2328.98</v>
+        <v>1879.05</v>
       </c>
       <c r="AA13" t="n">
-        <v>2413.98</v>
+        <v>1916.47</v>
       </c>
       <c r="AB13" t="n">
-        <v>2498.99</v>
+        <v>1953.89</v>
       </c>
       <c r="AC13" t="n">
-        <v>2584</v>
+        <v>1991.31</v>
       </c>
       <c r="AD13" t="n">
-        <v>2669.01</v>
+        <v>2028.74</v>
       </c>
       <c r="AE13" t="n">
-        <v>2754.02</v>
+        <v>2066.16</v>
       </c>
       <c r="AF13" t="n">
-        <v>2848.68</v>
+        <v>2103.58</v>
       </c>
       <c r="AG13" t="n">
-        <v>2943.34</v>
+        <v>2141</v>
       </c>
       <c r="AH13" t="n">
-        <v>3038</v>
+        <v>2178.43</v>
       </c>
       <c r="AI13" t="n">
-        <v>3132.66</v>
+        <v>2215.85</v>
       </c>
       <c r="AJ13" t="n">
-        <v>3227.32</v>
+        <v>2253.27</v>
       </c>
     </row>
     <row r="14">
@@ -2238,88 +2238,88 @@
         <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>19.46</v>
+        <v>20.33</v>
       </c>
       <c r="J14" t="n">
-        <v>19.63</v>
+        <v>21.29</v>
       </c>
       <c r="K14" t="n">
-        <v>19.99</v>
+        <v>22.45</v>
       </c>
       <c r="L14" t="n">
-        <v>19.99</v>
+        <v>23.24</v>
       </c>
       <c r="M14" t="n">
-        <v>19.99</v>
+        <v>24.03</v>
       </c>
       <c r="N14" t="n">
-        <v>19.99</v>
+        <v>24.83</v>
       </c>
       <c r="O14" t="n">
-        <v>19.99</v>
+        <v>25.62</v>
       </c>
       <c r="P14" t="n">
-        <v>19.99</v>
+        <v>26.42</v>
       </c>
       <c r="Q14" t="n">
-        <v>19.99</v>
+        <v>27.21</v>
       </c>
       <c r="R14" t="n">
-        <v>19.99</v>
+        <v>28.01</v>
       </c>
       <c r="S14" t="n">
-        <v>19.99</v>
+        <v>28.8</v>
       </c>
       <c r="T14" t="n">
-        <v>19.99</v>
+        <v>29.6</v>
       </c>
       <c r="U14" t="n">
-        <v>19.99</v>
+        <v>30.39</v>
       </c>
       <c r="V14" t="n">
-        <v>19.99</v>
+        <v>31.19</v>
       </c>
       <c r="W14" t="n">
-        <v>19.99</v>
+        <v>31.98</v>
       </c>
       <c r="X14" t="n">
-        <v>19.99</v>
+        <v>32.77</v>
       </c>
       <c r="Y14" t="n">
-        <v>19.99</v>
+        <v>33.57</v>
       </c>
       <c r="Z14" t="n">
-        <v>19.99</v>
+        <v>34.36</v>
       </c>
       <c r="AA14" t="n">
-        <v>20.13</v>
+        <v>35.16</v>
       </c>
       <c r="AB14" t="n">
-        <v>20.27</v>
+        <v>35.95</v>
       </c>
       <c r="AC14" t="n">
-        <v>20.41</v>
+        <v>36.75</v>
       </c>
       <c r="AD14" t="n">
-        <v>20.55</v>
+        <v>37.54</v>
       </c>
       <c r="AE14" t="n">
-        <v>20.69</v>
+        <v>38.34</v>
       </c>
       <c r="AF14" t="n">
-        <v>23.99</v>
+        <v>39.13</v>
       </c>
       <c r="AG14" t="n">
-        <v>27.29</v>
+        <v>39.93</v>
       </c>
       <c r="AH14" t="n">
-        <v>30.59</v>
+        <v>40.72</v>
       </c>
       <c r="AI14" t="n">
-        <v>33.88</v>
+        <v>41.51</v>
       </c>
       <c r="AJ14" t="n">
-        <v>37.18</v>
+        <v>42.31</v>
       </c>
     </row>
     <row r="15">
@@ -2362,88 +2362,88 @@
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>70.38</v>
+        <v>51.79</v>
       </c>
       <c r="J15" t="n">
-        <v>73.31999999999999</v>
+        <v>52.92</v>
       </c>
       <c r="K15" t="n">
-        <v>78.38</v>
+        <v>56.17</v>
       </c>
       <c r="L15" t="n">
-        <v>82.89</v>
+        <v>58.72</v>
       </c>
       <c r="M15" t="n">
-        <v>87.39</v>
+        <v>61.26</v>
       </c>
       <c r="N15" t="n">
-        <v>91.90000000000001</v>
+        <v>63.81</v>
       </c>
       <c r="O15" t="n">
-        <v>96.40000000000001</v>
+        <v>66.36</v>
       </c>
       <c r="P15" t="n">
-        <v>100.91</v>
+        <v>68.91</v>
       </c>
       <c r="Q15" t="n">
-        <v>105.61</v>
+        <v>71.45</v>
       </c>
       <c r="R15" t="n">
-        <v>110.31</v>
+        <v>74</v>
       </c>
       <c r="S15" t="n">
-        <v>115.02</v>
+        <v>76.55</v>
       </c>
       <c r="T15" t="n">
-        <v>119.72</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="U15" t="n">
-        <v>124.42</v>
+        <v>81.64</v>
       </c>
       <c r="V15" t="n">
-        <v>129.36</v>
+        <v>84.19</v>
       </c>
       <c r="W15" t="n">
-        <v>134.31</v>
+        <v>86.73999999999999</v>
       </c>
       <c r="X15" t="n">
-        <v>139.25</v>
+        <v>89.29000000000001</v>
       </c>
       <c r="Y15" t="n">
-        <v>144.19</v>
+        <v>91.84</v>
       </c>
       <c r="Z15" t="n">
-        <v>149.13</v>
+        <v>94.38</v>
       </c>
       <c r="AA15" t="n">
-        <v>154.46</v>
+        <v>96.93000000000001</v>
       </c>
       <c r="AB15" t="n">
-        <v>159.8</v>
+        <v>99.48</v>
       </c>
       <c r="AC15" t="n">
-        <v>165.13</v>
+        <v>102.03</v>
       </c>
       <c r="AD15" t="n">
-        <v>170.46</v>
+        <v>104.57</v>
       </c>
       <c r="AE15" t="n">
-        <v>175.79</v>
+        <v>107.12</v>
       </c>
       <c r="AF15" t="n">
-        <v>181.31</v>
+        <v>109.67</v>
       </c>
       <c r="AG15" t="n">
-        <v>186.83</v>
+        <v>112.22</v>
       </c>
       <c r="AH15" t="n">
-        <v>192.34</v>
+        <v>114.76</v>
       </c>
       <c r="AI15" t="n">
-        <v>197.86</v>
+        <v>117.31</v>
       </c>
       <c r="AJ15" t="n">
-        <v>203.38</v>
+        <v>119.86</v>
       </c>
     </row>
     <row r="16">
@@ -2486,88 +2486,88 @@
         <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>257.1</v>
+        <v>223.04</v>
       </c>
       <c r="J16" t="n">
-        <v>266.64</v>
+        <v>233.01</v>
       </c>
       <c r="K16" t="n">
-        <v>275.76</v>
+        <v>242.56</v>
       </c>
       <c r="L16" t="n">
-        <v>284.78</v>
+        <v>252.12</v>
       </c>
       <c r="M16" t="n">
-        <v>293.8</v>
+        <v>261.68</v>
       </c>
       <c r="N16" t="n">
-        <v>302.82</v>
+        <v>271.25</v>
       </c>
       <c r="O16" t="n">
-        <v>311.84</v>
+        <v>280.81</v>
       </c>
       <c r="P16" t="n">
-        <v>320.86</v>
+        <v>290.37</v>
       </c>
       <c r="Q16" t="n">
-        <v>329.98</v>
+        <v>299.94</v>
       </c>
       <c r="R16" t="n">
-        <v>339.1</v>
+        <v>309.5</v>
       </c>
       <c r="S16" t="n">
-        <v>348.22</v>
+        <v>319.07</v>
       </c>
       <c r="T16" t="n">
-        <v>357.34</v>
+        <v>328.63</v>
       </c>
       <c r="U16" t="n">
-        <v>366.46</v>
+        <v>338.19</v>
       </c>
       <c r="V16" t="n">
-        <v>376.03</v>
+        <v>347.76</v>
       </c>
       <c r="W16" t="n">
-        <v>385.61</v>
+        <v>357.32</v>
       </c>
       <c r="X16" t="n">
-        <v>395.19</v>
+        <v>366.88</v>
       </c>
       <c r="Y16" t="n">
-        <v>404.76</v>
+        <v>376.45</v>
       </c>
       <c r="Z16" t="n">
-        <v>414.34</v>
+        <v>386.01</v>
       </c>
       <c r="AA16" t="n">
-        <v>424.34</v>
+        <v>395.57</v>
       </c>
       <c r="AB16" t="n">
-        <v>434.34</v>
+        <v>405.14</v>
       </c>
       <c r="AC16" t="n">
-        <v>444.35</v>
+        <v>414.7</v>
       </c>
       <c r="AD16" t="n">
-        <v>454.35</v>
+        <v>424.26</v>
       </c>
       <c r="AE16" t="n">
-        <v>464.35</v>
+        <v>433.83</v>
       </c>
       <c r="AF16" t="n">
-        <v>474.63</v>
+        <v>443.39</v>
       </c>
       <c r="AG16" t="n">
-        <v>484.91</v>
+        <v>452.96</v>
       </c>
       <c r="AH16" t="n">
-        <v>495.18</v>
+        <v>462.52</v>
       </c>
       <c r="AI16" t="n">
-        <v>505.46</v>
+        <v>472.08</v>
       </c>
       <c r="AJ16" t="n">
-        <v>515.74</v>
+        <v>481.65</v>
       </c>
     </row>
     <row r="17">
@@ -2610,88 +2610,88 @@
         <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>-56.77</v>
+        <v>81.55</v>
       </c>
       <c r="J17" t="n">
-        <v>-4.97</v>
+        <v>145.53</v>
       </c>
       <c r="K17" t="n">
-        <v>-33.82</v>
+        <v>128.87</v>
       </c>
       <c r="L17" t="n">
-        <v>-33.82</v>
+        <v>141.05</v>
       </c>
       <c r="M17" t="n">
-        <v>-33.82</v>
+        <v>153.23</v>
       </c>
       <c r="N17" t="n">
-        <v>-33.82</v>
+        <v>165.41</v>
       </c>
       <c r="O17" t="n">
-        <v>-33.82</v>
+        <v>177.6</v>
       </c>
       <c r="P17" t="n">
-        <v>-33.82</v>
+        <v>189.78</v>
       </c>
       <c r="Q17" t="n">
-        <v>-33.82</v>
+        <v>201.96</v>
       </c>
       <c r="R17" t="n">
-        <v>-33.82</v>
+        <v>214.14</v>
       </c>
       <c r="S17" t="n">
-        <v>-33.82</v>
+        <v>226.33</v>
       </c>
       <c r="T17" t="n">
-        <v>-33.82</v>
+        <v>238.51</v>
       </c>
       <c r="U17" t="n">
-        <v>-33.82</v>
+        <v>250.69</v>
       </c>
       <c r="V17" t="n">
-        <v>-31.92</v>
+        <v>262.87</v>
       </c>
       <c r="W17" t="n">
-        <v>-30.01</v>
+        <v>275.06</v>
       </c>
       <c r="X17" t="n">
-        <v>-28.11</v>
+        <v>287.24</v>
       </c>
       <c r="Y17" t="n">
-        <v>-26.21</v>
+        <v>299.42</v>
       </c>
       <c r="Z17" t="n">
-        <v>-24.31</v>
+        <v>311.6</v>
       </c>
       <c r="AA17" t="n">
-        <v>-21.75</v>
+        <v>323.79</v>
       </c>
       <c r="AB17" t="n">
-        <v>-19.19</v>
+        <v>335.97</v>
       </c>
       <c r="AC17" t="n">
-        <v>-16.63</v>
+        <v>348.15</v>
       </c>
       <c r="AD17" t="n">
-        <v>-14.07</v>
+        <v>360.34</v>
       </c>
       <c r="AE17" t="n">
-        <v>-11.51</v>
+        <v>372.52</v>
       </c>
       <c r="AF17" t="n">
-        <v>-8.59</v>
+        <v>384.7</v>
       </c>
       <c r="AG17" t="n">
-        <v>-5.67</v>
+        <v>396.88</v>
       </c>
       <c r="AH17" t="n">
-        <v>-2.75</v>
+        <v>409.07</v>
       </c>
       <c r="AI17" t="n">
-        <v>0.17</v>
+        <v>421.25</v>
       </c>
       <c r="AJ17" t="n">
-        <v>3.09</v>
+        <v>433.43</v>
       </c>
     </row>
     <row r="18">
@@ -2734,88 +2734,88 @@
         <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>23.39</v>
+        <v>27.94</v>
       </c>
       <c r="J18" t="n">
-        <v>24.64</v>
+        <v>29.86</v>
       </c>
       <c r="K18" t="n">
-        <v>26.14</v>
+        <v>32.04</v>
       </c>
       <c r="L18" t="n">
-        <v>26.14</v>
+        <v>32.72</v>
       </c>
       <c r="M18" t="n">
-        <v>26.14</v>
+        <v>33.4</v>
       </c>
       <c r="N18" t="n">
-        <v>26.14</v>
+        <v>34.08</v>
       </c>
       <c r="O18" t="n">
-        <v>26.14</v>
+        <v>34.75</v>
       </c>
       <c r="P18" t="n">
-        <v>26.14</v>
+        <v>35.43</v>
       </c>
       <c r="Q18" t="n">
-        <v>26.14</v>
+        <v>36.11</v>
       </c>
       <c r="R18" t="n">
-        <v>26.14</v>
+        <v>36.79</v>
       </c>
       <c r="S18" t="n">
-        <v>26.14</v>
+        <v>37.47</v>
       </c>
       <c r="T18" t="n">
-        <v>26.14</v>
+        <v>38.14</v>
       </c>
       <c r="U18" t="n">
-        <v>26.14</v>
+        <v>38.82</v>
       </c>
       <c r="V18" t="n">
-        <v>26.2</v>
+        <v>39.5</v>
       </c>
       <c r="W18" t="n">
-        <v>26.26</v>
+        <v>40.18</v>
       </c>
       <c r="X18" t="n">
-        <v>26.32</v>
+        <v>40.86</v>
       </c>
       <c r="Y18" t="n">
-        <v>26.39</v>
+        <v>41.53</v>
       </c>
       <c r="Z18" t="n">
-        <v>26.45</v>
+        <v>42.21</v>
       </c>
       <c r="AA18" t="n">
-        <v>28.47</v>
+        <v>42.89</v>
       </c>
       <c r="AB18" t="n">
-        <v>30.49</v>
+        <v>43.57</v>
       </c>
       <c r="AC18" t="n">
-        <v>32.51</v>
+        <v>44.24</v>
       </c>
       <c r="AD18" t="n">
-        <v>34.53</v>
+        <v>44.92</v>
       </c>
       <c r="AE18" t="n">
-        <v>36.56</v>
+        <v>45.6</v>
       </c>
       <c r="AF18" t="n">
-        <v>38.8</v>
+        <v>46.28</v>
       </c>
       <c r="AG18" t="n">
-        <v>41.05</v>
+        <v>46.96</v>
       </c>
       <c r="AH18" t="n">
-        <v>43.29</v>
+        <v>47.63</v>
       </c>
       <c r="AI18" t="n">
-        <v>45.54</v>
+        <v>48.31</v>
       </c>
       <c r="AJ18" t="n">
-        <v>47.78</v>
+        <v>48.99</v>
       </c>
     </row>
     <row r="19">
@@ -2858,88 +2858,212 @@
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>48.9</v>
+        <v>50.51</v>
       </c>
       <c r="J19" t="n">
-        <v>37.48</v>
+        <v>40.18</v>
       </c>
       <c r="K19" t="n">
-        <v>40.7</v>
+        <v>44.5</v>
       </c>
       <c r="L19" t="n">
-        <v>40.7</v>
+        <v>45.59</v>
       </c>
       <c r="M19" t="n">
-        <v>40.7</v>
+        <v>46.68</v>
       </c>
       <c r="N19" t="n">
-        <v>40.7</v>
+        <v>47.78</v>
       </c>
       <c r="O19" t="n">
-        <v>40.7</v>
+        <v>48.87</v>
       </c>
       <c r="P19" t="n">
-        <v>40.7</v>
+        <v>49.97</v>
       </c>
       <c r="Q19" t="n">
-        <v>41.15</v>
+        <v>51.06</v>
       </c>
       <c r="R19" t="n">
-        <v>41.61</v>
+        <v>52.15</v>
       </c>
       <c r="S19" t="n">
-        <v>42.07</v>
+        <v>53.25</v>
       </c>
       <c r="T19" t="n">
-        <v>42.52</v>
+        <v>54.34</v>
       </c>
       <c r="U19" t="n">
-        <v>42.98</v>
+        <v>55.44</v>
       </c>
       <c r="V19" t="n">
-        <v>43.78</v>
+        <v>56.53</v>
       </c>
       <c r="W19" t="n">
-        <v>44.57</v>
+        <v>57.62</v>
       </c>
       <c r="X19" t="n">
-        <v>45.37</v>
+        <v>58.72</v>
       </c>
       <c r="Y19" t="n">
-        <v>46.17</v>
+        <v>59.81</v>
       </c>
       <c r="Z19" t="n">
-        <v>46.97</v>
+        <v>60.91</v>
       </c>
       <c r="AA19" t="n">
-        <v>47.81</v>
+        <v>62</v>
       </c>
       <c r="AB19" t="n">
-        <v>48.64</v>
+        <v>63.09</v>
       </c>
       <c r="AC19" t="n">
-        <v>49.48</v>
+        <v>64.19</v>
       </c>
       <c r="AD19" t="n">
-        <v>50.31</v>
+        <v>65.28</v>
       </c>
       <c r="AE19" t="n">
-        <v>51.15</v>
+        <v>66.38</v>
       </c>
       <c r="AF19" t="n">
-        <v>52</v>
+        <v>67.47</v>
       </c>
       <c r="AG19" t="n">
-        <v>52.85</v>
+        <v>68.56</v>
       </c>
       <c r="AH19" t="n">
-        <v>53.7</v>
+        <v>69.66</v>
       </c>
       <c r="AI19" t="n">
-        <v>54.54</v>
+        <v>70.75</v>
       </c>
       <c r="AJ19" t="n">
-        <v>55.39</v>
+        <v>71.84999999999999</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Demand</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ELCHTIXX03</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Output demand of dispatch-ready in Haiti</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>not needed</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>not needed</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>not needed</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>User defined</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="J20" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="K20" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="L20" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="M20" t="n">
+        <v>3.53</v>
+      </c>
+      <c r="N20" t="n">
+        <v>3.63</v>
+      </c>
+      <c r="O20" t="n">
+        <v>3.73</v>
+      </c>
+      <c r="P20" t="n">
+        <v>3.83</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>3.93</v>
+      </c>
+      <c r="R20" t="n">
+        <v>4.03</v>
+      </c>
+      <c r="S20" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="T20" t="n">
+        <v>4.23</v>
+      </c>
+      <c r="U20" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="V20" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="W20" t="n">
+        <v>4.53</v>
+      </c>
+      <c r="X20" t="n">
+        <v>4.63</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>4.73</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>4.83</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>4.93</v>
+      </c>
+      <c r="AB20" t="n">
+        <v>5.03</v>
+      </c>
+      <c r="AC20" t="n">
+        <v>5.13</v>
+      </c>
+      <c r="AD20" t="n">
+        <v>5.23</v>
+      </c>
+      <c r="AE20" t="n">
+        <v>5.34</v>
+      </c>
+      <c r="AF20" t="n">
+        <v>5.44</v>
+      </c>
+      <c r="AG20" t="n">
+        <v>5.54</v>
+      </c>
+      <c r="AH20" t="n">
+        <v>5.64</v>
+      </c>
+      <c r="AI20" t="n">
+        <v>5.74</v>
+      </c>
+      <c r="AJ20" t="n">
+        <v>5.84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix double-counting of CCG00/CCG01 in A3 gas aggregation and restore original OG inputs
A3 was summing both suffix variants (00 and 01) when aggregating
CCG+OCG → NGS, causing doubled ResidualCapacity for ARG, BRA, MEX.
Added two-stage aggregation: deduplicate within same base tech (max)
before summing across different techs (CCG+OCG).

Also restores OG_csvs_inputs to original state with 00/01 suffixes
and updates A1_Outputs after re-running A3 migration.
</commit_message>
<xml_diff>
--- a/t1_confection/A1_Outputs/A1_Outputs_BAU/A-O_Demand.xlsx
+++ b/t1_confection/A1_Outputs/A1_Outputs_BAU/A-O_Demand.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ20"/>
+  <dimension ref="A1:AJ19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.85546875" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
@@ -750,88 +750,88 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>524.49</v>
+        <v>555.91</v>
       </c>
       <c r="J2" t="n">
-        <v>506.39</v>
+        <v>555.91</v>
       </c>
       <c r="K2" t="n">
-        <v>509.61</v>
+        <v>555.91</v>
       </c>
       <c r="L2" t="n">
-        <v>513.74</v>
+        <v>567.9</v>
       </c>
       <c r="M2" t="n">
-        <v>517.87</v>
+        <v>579.88</v>
       </c>
       <c r="N2" t="n">
-        <v>522</v>
+        <v>591.87</v>
       </c>
       <c r="O2" t="n">
-        <v>526.13</v>
+        <v>603.85</v>
       </c>
       <c r="P2" t="n">
-        <v>530.25</v>
+        <v>615.83</v>
       </c>
       <c r="Q2" t="n">
-        <v>534.38</v>
+        <v>630.22</v>
       </c>
       <c r="R2" t="n">
-        <v>538.51</v>
+        <v>644.61</v>
       </c>
       <c r="S2" t="n">
-        <v>542.64</v>
+        <v>659</v>
       </c>
       <c r="T2" t="n">
-        <v>546.77</v>
+        <v>673.38</v>
       </c>
       <c r="U2" t="n">
-        <v>550.9</v>
+        <v>687.77</v>
       </c>
       <c r="V2" t="n">
-        <v>555.03</v>
+        <v>703</v>
       </c>
       <c r="W2" t="n">
-        <v>559.16</v>
+        <v>718.23</v>
       </c>
       <c r="X2" t="n">
-        <v>563.29</v>
+        <v>733.46</v>
       </c>
       <c r="Y2" t="n">
-        <v>567.42</v>
+        <v>748.7</v>
       </c>
       <c r="Z2" t="n">
-        <v>571.55</v>
+        <v>763.9299999999999</v>
       </c>
       <c r="AA2" t="n">
-        <v>575.6799999999999</v>
+        <v>778.8099999999999</v>
       </c>
       <c r="AB2" t="n">
-        <v>579.8099999999999</v>
+        <v>793.6900000000001</v>
       </c>
       <c r="AC2" t="n">
-        <v>583.9299999999999</v>
+        <v>808.58</v>
       </c>
       <c r="AD2" t="n">
-        <v>588.0599999999999</v>
+        <v>823.46</v>
       </c>
       <c r="AE2" t="n">
-        <v>592.1900000000001</v>
+        <v>838.34</v>
       </c>
       <c r="AF2" t="n">
-        <v>596.3200000000001</v>
+        <v>853.52</v>
       </c>
       <c r="AG2" t="n">
-        <v>600.45</v>
+        <v>868.7</v>
       </c>
       <c r="AH2" t="n">
-        <v>604.58</v>
+        <v>883.88</v>
       </c>
       <c r="AI2" t="n">
-        <v>608.71</v>
+        <v>899.0599999999999</v>
       </c>
       <c r="AJ2" t="n">
-        <v>612.84</v>
+        <v>914.23</v>
       </c>
     </row>
     <row r="3">
@@ -874,88 +874,88 @@
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>42.81</v>
+        <v>48.49</v>
       </c>
       <c r="J3" t="n">
-        <v>45.15</v>
+        <v>50.57</v>
       </c>
       <c r="K3" t="n">
-        <v>48.39</v>
+        <v>52.65</v>
       </c>
       <c r="L3" t="n">
-        <v>51.14</v>
+        <v>55.07</v>
       </c>
       <c r="M3" t="n">
-        <v>53.88</v>
+        <v>57.49</v>
       </c>
       <c r="N3" t="n">
-        <v>56.63</v>
+        <v>59.92</v>
       </c>
       <c r="O3" t="n">
-        <v>59.38</v>
+        <v>62.34</v>
       </c>
       <c r="P3" t="n">
-        <v>62.13</v>
+        <v>64.76000000000001</v>
       </c>
       <c r="Q3" t="n">
-        <v>64.88</v>
+        <v>67.45999999999999</v>
       </c>
       <c r="R3" t="n">
-        <v>67.63</v>
+        <v>70.16</v>
       </c>
       <c r="S3" t="n">
-        <v>70.37</v>
+        <v>72.84999999999999</v>
       </c>
       <c r="T3" t="n">
-        <v>73.12</v>
+        <v>75.55</v>
       </c>
       <c r="U3" t="n">
-        <v>75.87</v>
+        <v>78.25</v>
       </c>
       <c r="V3" t="n">
-        <v>78.62</v>
+        <v>81.34</v>
       </c>
       <c r="W3" t="n">
-        <v>81.37</v>
+        <v>84.43000000000001</v>
       </c>
       <c r="X3" t="n">
-        <v>84.12</v>
+        <v>87.52</v>
       </c>
       <c r="Y3" t="n">
-        <v>86.87</v>
+        <v>90.61</v>
       </c>
       <c r="Z3" t="n">
-        <v>89.61</v>
+        <v>93.7</v>
       </c>
       <c r="AA3" t="n">
-        <v>92.36</v>
+        <v>97.23</v>
       </c>
       <c r="AB3" t="n">
-        <v>95.11</v>
+        <v>100.76</v>
       </c>
       <c r="AC3" t="n">
-        <v>97.86</v>
+        <v>104.29</v>
       </c>
       <c r="AD3" t="n">
-        <v>100.61</v>
+        <v>107.82</v>
       </c>
       <c r="AE3" t="n">
-        <v>103.36</v>
+        <v>111.35</v>
       </c>
       <c r="AF3" t="n">
-        <v>106.1</v>
+        <v>115.41</v>
       </c>
       <c r="AG3" t="n">
-        <v>108.85</v>
+        <v>119.46</v>
       </c>
       <c r="AH3" t="n">
-        <v>111.6</v>
+        <v>123.52</v>
       </c>
       <c r="AI3" t="n">
-        <v>114.35</v>
+        <v>127.58</v>
       </c>
       <c r="AJ3" t="n">
-        <v>117.1</v>
+        <v>131.63</v>
       </c>
     </row>
     <row r="4">
@@ -998,88 +998,88 @@
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>2599.63</v>
+        <v>2217.88</v>
       </c>
       <c r="J4" t="n">
-        <v>2637.58</v>
+        <v>2217.88</v>
       </c>
       <c r="K4" t="n">
-        <v>2719.49</v>
+        <v>2217.88</v>
       </c>
       <c r="L4" t="n">
-        <v>2775.31</v>
+        <v>2217.88</v>
       </c>
       <c r="M4" t="n">
-        <v>2831.14</v>
+        <v>2217.88</v>
       </c>
       <c r="N4" t="n">
-        <v>2886.97</v>
+        <v>2217.88</v>
       </c>
       <c r="O4" t="n">
-        <v>2942.8</v>
+        <v>2217.88</v>
       </c>
       <c r="P4" t="n">
-        <v>2998.63</v>
+        <v>2217.88</v>
       </c>
       <c r="Q4" t="n">
-        <v>3054.45</v>
+        <v>2239.39</v>
       </c>
       <c r="R4" t="n">
-        <v>3110.28</v>
+        <v>2260.91</v>
       </c>
       <c r="S4" t="n">
-        <v>3166.11</v>
+        <v>2282.45</v>
       </c>
       <c r="T4" t="n">
-        <v>3221.94</v>
+        <v>2303.96</v>
       </c>
       <c r="U4" t="n">
-        <v>3277.77</v>
+        <v>2325.48</v>
       </c>
       <c r="V4" t="n">
-        <v>3333.59</v>
+        <v>2365.7</v>
       </c>
       <c r="W4" t="n">
-        <v>3389.42</v>
+        <v>2405.95</v>
       </c>
       <c r="X4" t="n">
-        <v>3445.25</v>
+        <v>2446.19</v>
       </c>
       <c r="Y4" t="n">
-        <v>3501.08</v>
+        <v>2486.43</v>
       </c>
       <c r="Z4" t="n">
-        <v>3556.91</v>
+        <v>2526.68</v>
       </c>
       <c r="AA4" t="n">
-        <v>3612.74</v>
+        <v>2565.7</v>
       </c>
       <c r="AB4" t="n">
-        <v>3668.56</v>
+        <v>2604.71</v>
       </c>
       <c r="AC4" t="n">
-        <v>3724.39</v>
+        <v>2643.73</v>
       </c>
       <c r="AD4" t="n">
-        <v>3780.22</v>
+        <v>2682.73</v>
       </c>
       <c r="AE4" t="n">
-        <v>3836.05</v>
+        <v>2721.76</v>
       </c>
       <c r="AF4" t="n">
-        <v>3891.88</v>
+        <v>2761.04</v>
       </c>
       <c r="AG4" t="n">
-        <v>3947.7</v>
+        <v>2800.31</v>
       </c>
       <c r="AH4" t="n">
-        <v>4003.53</v>
+        <v>2839.59</v>
       </c>
       <c r="AI4" t="n">
-        <v>4059.36</v>
+        <v>2878.87</v>
       </c>
       <c r="AJ4" t="n">
-        <v>4115.19</v>
+        <v>2918.15</v>
       </c>
     </row>
     <row r="5">
@@ -1122,88 +1122,88 @@
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>3.87</v>
+        <v>14.87</v>
       </c>
       <c r="J5" t="n">
-        <v>4.12</v>
+        <v>14.87</v>
       </c>
       <c r="K5" t="n">
-        <v>4.37</v>
+        <v>14.87</v>
       </c>
       <c r="L5" t="n">
-        <v>4.62</v>
+        <v>14.87</v>
       </c>
       <c r="M5" t="n">
-        <v>4.86</v>
+        <v>14.87</v>
       </c>
       <c r="N5" t="n">
-        <v>5.11</v>
+        <v>14.87</v>
       </c>
       <c r="O5" t="n">
-        <v>5.36</v>
+        <v>14.87</v>
       </c>
       <c r="P5" t="n">
-        <v>5.6</v>
+        <v>14.87</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.85</v>
+        <v>14.87</v>
       </c>
       <c r="R5" t="n">
-        <v>6.1</v>
+        <v>14.87</v>
       </c>
       <c r="S5" t="n">
-        <v>6.35</v>
+        <v>14.87</v>
       </c>
       <c r="T5" t="n">
-        <v>6.59</v>
+        <v>14.87</v>
       </c>
       <c r="U5" t="n">
-        <v>6.84</v>
+        <v>14.87</v>
       </c>
       <c r="V5" t="n">
-        <v>7.09</v>
+        <v>14.87</v>
       </c>
       <c r="W5" t="n">
-        <v>7.33</v>
+        <v>14.87</v>
       </c>
       <c r="X5" t="n">
-        <v>7.58</v>
+        <v>14.87</v>
       </c>
       <c r="Y5" t="n">
-        <v>7.83</v>
+        <v>14.87</v>
       </c>
       <c r="Z5" t="n">
-        <v>8.08</v>
+        <v>14.87</v>
       </c>
       <c r="AA5" t="n">
-        <v>8.32</v>
+        <v>14.88</v>
       </c>
       <c r="AB5" t="n">
-        <v>8.57</v>
+        <v>14.88</v>
       </c>
       <c r="AC5" t="n">
-        <v>8.82</v>
+        <v>14.89</v>
       </c>
       <c r="AD5" t="n">
-        <v>9.06</v>
+        <v>14.9</v>
       </c>
       <c r="AE5" t="n">
-        <v>9.31</v>
+        <v>14.9</v>
       </c>
       <c r="AF5" t="n">
-        <v>9.56</v>
+        <v>15.73</v>
       </c>
       <c r="AG5" t="n">
-        <v>9.81</v>
+        <v>16.55</v>
       </c>
       <c r="AH5" t="n">
-        <v>10.05</v>
+        <v>17.37</v>
       </c>
       <c r="AI5" t="n">
-        <v>10.3</v>
+        <v>18.19</v>
       </c>
       <c r="AJ5" t="n">
-        <v>10.55</v>
+        <v>19.02</v>
       </c>
     </row>
     <row r="6">
@@ -1246,88 +1246,88 @@
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>302.25</v>
+        <v>271.4</v>
       </c>
       <c r="J6" t="n">
-        <v>318.54</v>
+        <v>271.4</v>
       </c>
       <c r="K6" t="n">
-        <v>334.66</v>
+        <v>271.4</v>
       </c>
       <c r="L6" t="n">
-        <v>350.81</v>
+        <v>271.4</v>
       </c>
       <c r="M6" t="n">
-        <v>366.95</v>
+        <v>271.4</v>
       </c>
       <c r="N6" t="n">
-        <v>383.1</v>
+        <v>271.4</v>
       </c>
       <c r="O6" t="n">
-        <v>399.25</v>
+        <v>271.4</v>
       </c>
       <c r="P6" t="n">
-        <v>415.4</v>
+        <v>271.4</v>
       </c>
       <c r="Q6" t="n">
-        <v>431.54</v>
+        <v>272.9</v>
       </c>
       <c r="R6" t="n">
-        <v>447.69</v>
+        <v>274.4</v>
       </c>
       <c r="S6" t="n">
-        <v>463.84</v>
+        <v>275.89</v>
       </c>
       <c r="T6" t="n">
-        <v>479.99</v>
+        <v>277.39</v>
       </c>
       <c r="U6" t="n">
-        <v>496.14</v>
+        <v>278.88</v>
       </c>
       <c r="V6" t="n">
-        <v>512.28</v>
+        <v>284.94</v>
       </c>
       <c r="W6" t="n">
-        <v>528.4299999999999</v>
+        <v>291</v>
       </c>
       <c r="X6" t="n">
-        <v>544.58</v>
+        <v>297.06</v>
       </c>
       <c r="Y6" t="n">
-        <v>560.73</v>
+        <v>303.12</v>
       </c>
       <c r="Z6" t="n">
-        <v>576.87</v>
+        <v>309.19</v>
       </c>
       <c r="AA6" t="n">
-        <v>593.02</v>
+        <v>315.49</v>
       </c>
       <c r="AB6" t="n">
-        <v>609.17</v>
+        <v>321.79</v>
       </c>
       <c r="AC6" t="n">
-        <v>625.3200000000001</v>
+        <v>328.1</v>
       </c>
       <c r="AD6" t="n">
-        <v>641.47</v>
+        <v>334.4</v>
       </c>
       <c r="AE6" t="n">
-        <v>657.61</v>
+        <v>340.71</v>
       </c>
       <c r="AF6" t="n">
-        <v>673.76</v>
+        <v>347</v>
       </c>
       <c r="AG6" t="n">
-        <v>689.91</v>
+        <v>353.29</v>
       </c>
       <c r="AH6" t="n">
-        <v>706.0599999999999</v>
+        <v>359.58</v>
       </c>
       <c r="AI6" t="n">
-        <v>722.2</v>
+        <v>365.87</v>
       </c>
       <c r="AJ6" t="n">
-        <v>738.35</v>
+        <v>372.16</v>
       </c>
     </row>
     <row r="7">
@@ -1370,88 +1370,88 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>288.23</v>
+        <v>383.28</v>
       </c>
       <c r="J7" t="n">
-        <v>296.14</v>
+        <v>393.61</v>
       </c>
       <c r="K7" t="n">
-        <v>310.83</v>
+        <v>403.93</v>
       </c>
       <c r="L7" t="n">
-        <v>321.53</v>
+        <v>415.72</v>
       </c>
       <c r="M7" t="n">
-        <v>332.24</v>
+        <v>427.5</v>
       </c>
       <c r="N7" t="n">
-        <v>342.94</v>
+        <v>439.29</v>
       </c>
       <c r="O7" t="n">
-        <v>353.65</v>
+        <v>451.08</v>
       </c>
       <c r="P7" t="n">
-        <v>364.35</v>
+        <v>462.86</v>
       </c>
       <c r="Q7" t="n">
-        <v>375.05</v>
+        <v>475.69</v>
       </c>
       <c r="R7" t="n">
-        <v>385.76</v>
+        <v>488.52</v>
       </c>
       <c r="S7" t="n">
-        <v>396.46</v>
+        <v>501.35</v>
       </c>
       <c r="T7" t="n">
-        <v>407.17</v>
+        <v>514.17</v>
       </c>
       <c r="U7" t="n">
-        <v>417.87</v>
+        <v>527</v>
       </c>
       <c r="V7" t="n">
-        <v>428.58</v>
+        <v>541.29</v>
       </c>
       <c r="W7" t="n">
-        <v>439.28</v>
+        <v>555.58</v>
       </c>
       <c r="X7" t="n">
-        <v>449.98</v>
+        <v>569.86</v>
       </c>
       <c r="Y7" t="n">
-        <v>460.69</v>
+        <v>584.15</v>
       </c>
       <c r="Z7" t="n">
-        <v>471.39</v>
+        <v>598.4400000000001</v>
       </c>
       <c r="AA7" t="n">
-        <v>482.1</v>
+        <v>614</v>
       </c>
       <c r="AB7" t="n">
-        <v>492.8</v>
+        <v>629.5599999999999</v>
       </c>
       <c r="AC7" t="n">
-        <v>503.51</v>
+        <v>645.13</v>
       </c>
       <c r="AD7" t="n">
-        <v>514.21</v>
+        <v>660.6900000000001</v>
       </c>
       <c r="AE7" t="n">
-        <v>524.91</v>
+        <v>676.26</v>
       </c>
       <c r="AF7" t="n">
-        <v>535.62</v>
+        <v>692.9400000000001</v>
       </c>
       <c r="AG7" t="n">
-        <v>546.3200000000001</v>
+        <v>709.63</v>
       </c>
       <c r="AH7" t="n">
-        <v>557.03</v>
+        <v>726.3099999999999</v>
       </c>
       <c r="AI7" t="n">
-        <v>567.73</v>
+        <v>743</v>
       </c>
       <c r="AJ7" t="n">
-        <v>578.4400000000001</v>
+        <v>759.6799999999999</v>
       </c>
     </row>
     <row r="8">
@@ -1494,88 +1494,88 @@
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>44.28</v>
+        <v>45.41</v>
       </c>
       <c r="J8" t="n">
-        <v>44.68</v>
+        <v>47.7</v>
       </c>
       <c r="K8" t="n">
-        <v>43.57</v>
+        <v>50</v>
       </c>
       <c r="L8" t="n">
-        <v>44.46</v>
+        <v>52.7</v>
       </c>
       <c r="M8" t="n">
-        <v>45.34</v>
+        <v>55.41</v>
       </c>
       <c r="N8" t="n">
-        <v>46.23</v>
+        <v>58.11</v>
       </c>
       <c r="O8" t="n">
-        <v>47.12</v>
+        <v>60.82</v>
       </c>
       <c r="P8" t="n">
-        <v>48</v>
+        <v>63.53</v>
       </c>
       <c r="Q8" t="n">
-        <v>48.89</v>
+        <v>66.48999999999999</v>
       </c>
       <c r="R8" t="n">
-        <v>49.77</v>
+        <v>69.45</v>
       </c>
       <c r="S8" t="n">
-        <v>50.66</v>
+        <v>72.41</v>
       </c>
       <c r="T8" t="n">
-        <v>51.54</v>
+        <v>75.37</v>
       </c>
       <c r="U8" t="n">
-        <v>52.43</v>
+        <v>78.33</v>
       </c>
       <c r="V8" t="n">
-        <v>53.31</v>
+        <v>81.68000000000001</v>
       </c>
       <c r="W8" t="n">
-        <v>54.2</v>
+        <v>85.03</v>
       </c>
       <c r="X8" t="n">
-        <v>55.08</v>
+        <v>88.37</v>
       </c>
       <c r="Y8" t="n">
-        <v>55.97</v>
+        <v>91.72</v>
       </c>
       <c r="Z8" t="n">
-        <v>56.86</v>
+        <v>95.06999999999999</v>
       </c>
       <c r="AA8" t="n">
-        <v>57.74</v>
+        <v>98.70999999999999</v>
       </c>
       <c r="AB8" t="n">
-        <v>58.63</v>
+        <v>102.36</v>
       </c>
       <c r="AC8" t="n">
-        <v>59.51</v>
+        <v>106</v>
       </c>
       <c r="AD8" t="n">
-        <v>60.4</v>
+        <v>109.64</v>
       </c>
       <c r="AE8" t="n">
-        <v>61.28</v>
+        <v>113.29</v>
       </c>
       <c r="AF8" t="n">
-        <v>62.17</v>
+        <v>117.13</v>
       </c>
       <c r="AG8" t="n">
-        <v>63.05</v>
+        <v>120.96</v>
       </c>
       <c r="AH8" t="n">
-        <v>63.94</v>
+        <v>124.8</v>
       </c>
       <c r="AI8" t="n">
-        <v>64.81999999999999</v>
+        <v>128.64</v>
       </c>
       <c r="AJ8" t="n">
-        <v>65.70999999999999</v>
+        <v>132.47</v>
       </c>
     </row>
     <row r="9">
@@ -1618,88 +1618,88 @@
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>86.09</v>
+        <v>66.8</v>
       </c>
       <c r="J9" t="n">
-        <v>89.09999999999999</v>
+        <v>66.92</v>
       </c>
       <c r="K9" t="n">
-        <v>92.11</v>
+        <v>67.03</v>
       </c>
       <c r="L9" t="n">
-        <v>95.12</v>
+        <v>71.7</v>
       </c>
       <c r="M9" t="n">
-        <v>98.14</v>
+        <v>76.37</v>
       </c>
       <c r="N9" t="n">
-        <v>101.15</v>
+        <v>81.04000000000001</v>
       </c>
       <c r="O9" t="n">
-        <v>104.16</v>
+        <v>85.7</v>
       </c>
       <c r="P9" t="n">
-        <v>107.18</v>
+        <v>90.37</v>
       </c>
       <c r="Q9" t="n">
-        <v>110.19</v>
+        <v>95.44</v>
       </c>
       <c r="R9" t="n">
-        <v>113.2</v>
+        <v>100.51</v>
       </c>
       <c r="S9" t="n">
-        <v>116.21</v>
+        <v>105.58</v>
       </c>
       <c r="T9" t="n">
-        <v>119.23</v>
+        <v>110.65</v>
       </c>
       <c r="U9" t="n">
-        <v>122.24</v>
+        <v>115.72</v>
       </c>
       <c r="V9" t="n">
-        <v>125.25</v>
+        <v>121.48</v>
       </c>
       <c r="W9" t="n">
-        <v>128.27</v>
+        <v>127.23</v>
       </c>
       <c r="X9" t="n">
-        <v>131.28</v>
+        <v>132.98</v>
       </c>
       <c r="Y9" t="n">
-        <v>134.29</v>
+        <v>138.73</v>
       </c>
       <c r="Z9" t="n">
-        <v>137.31</v>
+        <v>144.49</v>
       </c>
       <c r="AA9" t="n">
-        <v>140.32</v>
+        <v>150.83</v>
       </c>
       <c r="AB9" t="n">
-        <v>143.33</v>
+        <v>157.18</v>
       </c>
       <c r="AC9" t="n">
-        <v>146.34</v>
+        <v>163.53</v>
       </c>
       <c r="AD9" t="n">
-        <v>149.36</v>
+        <v>169.88</v>
       </c>
       <c r="AE9" t="n">
-        <v>152.37</v>
+        <v>176.23</v>
       </c>
       <c r="AF9" t="n">
-        <v>155.38</v>
+        <v>183.07</v>
       </c>
       <c r="AG9" t="n">
-        <v>158.4</v>
+        <v>189.91</v>
       </c>
       <c r="AH9" t="n">
-        <v>161.41</v>
+        <v>196.75</v>
       </c>
       <c r="AI9" t="n">
-        <v>164.42</v>
+        <v>203.59</v>
       </c>
       <c r="AJ9" t="n">
-        <v>167.44</v>
+        <v>210.44</v>
       </c>
     </row>
     <row r="10">
@@ -1742,88 +1742,88 @@
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>129.57</v>
+        <v>97.41</v>
       </c>
       <c r="J10" t="n">
-        <v>137.75</v>
+        <v>98.33</v>
       </c>
       <c r="K10" t="n">
-        <v>139.6</v>
+        <v>99.26000000000001</v>
       </c>
       <c r="L10" t="n">
-        <v>145.41</v>
+        <v>102.44</v>
       </c>
       <c r="M10" t="n">
-        <v>151.21</v>
+        <v>105.63</v>
       </c>
       <c r="N10" t="n">
-        <v>157.02</v>
+        <v>108.81</v>
       </c>
       <c r="O10" t="n">
-        <v>162.82</v>
+        <v>111.99</v>
       </c>
       <c r="P10" t="n">
-        <v>168.63</v>
+        <v>115.18</v>
       </c>
       <c r="Q10" t="n">
-        <v>174.43</v>
+        <v>118.64</v>
       </c>
       <c r="R10" t="n">
-        <v>180.24</v>
+        <v>122.11</v>
       </c>
       <c r="S10" t="n">
-        <v>186.04</v>
+        <v>125.58</v>
       </c>
       <c r="T10" t="n">
-        <v>191.85</v>
+        <v>129.04</v>
       </c>
       <c r="U10" t="n">
-        <v>197.65</v>
+        <v>132.51</v>
       </c>
       <c r="V10" t="n">
-        <v>203.46</v>
+        <v>136.51</v>
       </c>
       <c r="W10" t="n">
-        <v>209.26</v>
+        <v>140.51</v>
       </c>
       <c r="X10" t="n">
-        <v>215.07</v>
+        <v>144.51</v>
       </c>
       <c r="Y10" t="n">
-        <v>220.87</v>
+        <v>148.52</v>
       </c>
       <c r="Z10" t="n">
-        <v>226.68</v>
+        <v>152.52</v>
       </c>
       <c r="AA10" t="n">
-        <v>232.48</v>
+        <v>157.16</v>
       </c>
       <c r="AB10" t="n">
-        <v>238.29</v>
+        <v>161.81</v>
       </c>
       <c r="AC10" t="n">
-        <v>244.09</v>
+        <v>166.46</v>
       </c>
       <c r="AD10" t="n">
-        <v>249.9</v>
+        <v>171.1</v>
       </c>
       <c r="AE10" t="n">
-        <v>255.7</v>
+        <v>175.75</v>
       </c>
       <c r="AF10" t="n">
-        <v>261.51</v>
+        <v>181.04</v>
       </c>
       <c r="AG10" t="n">
-        <v>267.31</v>
+        <v>186.33</v>
       </c>
       <c r="AH10" t="n">
-        <v>273.12</v>
+        <v>191.61</v>
       </c>
       <c r="AI10" t="n">
-        <v>278.92</v>
+        <v>196.9</v>
       </c>
       <c r="AJ10" t="n">
-        <v>284.73</v>
+        <v>202.19</v>
       </c>
     </row>
     <row r="11">
@@ -1866,88 +1866,88 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>47.17</v>
+        <v>38.02</v>
       </c>
       <c r="J11" t="n">
-        <v>48.54</v>
+        <v>38.02</v>
       </c>
       <c r="K11" t="n">
-        <v>48.53</v>
+        <v>38.02</v>
       </c>
       <c r="L11" t="n">
-        <v>50.07</v>
+        <v>38.02</v>
       </c>
       <c r="M11" t="n">
-        <v>51.6</v>
+        <v>38.02</v>
       </c>
       <c r="N11" t="n">
-        <v>53.13</v>
+        <v>38.02</v>
       </c>
       <c r="O11" t="n">
-        <v>54.66</v>
+        <v>38.02</v>
       </c>
       <c r="P11" t="n">
-        <v>56.19</v>
+        <v>38.02</v>
       </c>
       <c r="Q11" t="n">
-        <v>57.72</v>
+        <v>38.02</v>
       </c>
       <c r="R11" t="n">
-        <v>59.25</v>
+        <v>38.02</v>
       </c>
       <c r="S11" t="n">
-        <v>60.79</v>
+        <v>38.02</v>
       </c>
       <c r="T11" t="n">
-        <v>62.32</v>
+        <v>38.02</v>
       </c>
       <c r="U11" t="n">
-        <v>63.85</v>
+        <v>38.02</v>
       </c>
       <c r="V11" t="n">
-        <v>65.38</v>
+        <v>40.54</v>
       </c>
       <c r="W11" t="n">
-        <v>66.91</v>
+        <v>43.06</v>
       </c>
       <c r="X11" t="n">
-        <v>68.44</v>
+        <v>45.58</v>
       </c>
       <c r="Y11" t="n">
-        <v>69.97</v>
+        <v>48.09</v>
       </c>
       <c r="Z11" t="n">
-        <v>71.5</v>
+        <v>50.61</v>
       </c>
       <c r="AA11" t="n">
-        <v>73.04000000000001</v>
+        <v>59</v>
       </c>
       <c r="AB11" t="n">
-        <v>74.56999999999999</v>
+        <v>67.38</v>
       </c>
       <c r="AC11" t="n">
-        <v>76.09999999999999</v>
+        <v>75.77</v>
       </c>
       <c r="AD11" t="n">
-        <v>77.63</v>
+        <v>84.15000000000001</v>
       </c>
       <c r="AE11" t="n">
-        <v>79.16</v>
+        <v>92.54000000000001</v>
       </c>
       <c r="AF11" t="n">
-        <v>80.69</v>
+        <v>103.19</v>
       </c>
       <c r="AG11" t="n">
-        <v>82.22</v>
+        <v>113.85</v>
       </c>
       <c r="AH11" t="n">
-        <v>83.75</v>
+        <v>124.51</v>
       </c>
       <c r="AI11" t="n">
-        <v>85.29000000000001</v>
+        <v>135.16</v>
       </c>
       <c r="AJ11" t="n">
-        <v>86.81999999999999</v>
+        <v>145.82</v>
       </c>
     </row>
     <row r="12">
@@ -1990,88 +1990,88 @@
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>43.14</v>
+        <v>32.8</v>
       </c>
       <c r="J12" t="n">
-        <v>44.46</v>
+        <v>32.8</v>
       </c>
       <c r="K12" t="n">
-        <v>45.94</v>
+        <v>32.8</v>
       </c>
       <c r="L12" t="n">
-        <v>47.24</v>
+        <v>32.8</v>
       </c>
       <c r="M12" t="n">
-        <v>48.55</v>
+        <v>32.8</v>
       </c>
       <c r="N12" t="n">
-        <v>49.85</v>
+        <v>32.8</v>
       </c>
       <c r="O12" t="n">
-        <v>51.16</v>
+        <v>32.8</v>
       </c>
       <c r="P12" t="n">
-        <v>52.46</v>
+        <v>32.8</v>
       </c>
       <c r="Q12" t="n">
-        <v>53.77</v>
+        <v>32.8</v>
       </c>
       <c r="R12" t="n">
-        <v>55.07</v>
+        <v>32.8</v>
       </c>
       <c r="S12" t="n">
-        <v>56.38</v>
+        <v>32.8</v>
       </c>
       <c r="T12" t="n">
-        <v>57.68</v>
+        <v>32.8</v>
       </c>
       <c r="U12" t="n">
-        <v>58.98</v>
+        <v>32.8</v>
       </c>
       <c r="V12" t="n">
-        <v>60.29</v>
+        <v>32.8</v>
       </c>
       <c r="W12" t="n">
-        <v>61.59</v>
+        <v>32.8</v>
       </c>
       <c r="X12" t="n">
-        <v>62.9</v>
+        <v>32.8</v>
       </c>
       <c r="Y12" t="n">
-        <v>64.2</v>
+        <v>32.8</v>
       </c>
       <c r="Z12" t="n">
-        <v>65.51000000000001</v>
+        <v>32.8</v>
       </c>
       <c r="AA12" t="n">
-        <v>66.81</v>
+        <v>32.8</v>
       </c>
       <c r="AB12" t="n">
-        <v>68.12</v>
+        <v>32.8</v>
       </c>
       <c r="AC12" t="n">
-        <v>69.42</v>
+        <v>32.8</v>
       </c>
       <c r="AD12" t="n">
-        <v>70.73</v>
+        <v>32.8</v>
       </c>
       <c r="AE12" t="n">
-        <v>72.03</v>
+        <v>32.8</v>
       </c>
       <c r="AF12" t="n">
-        <v>73.34</v>
+        <v>37.49</v>
       </c>
       <c r="AG12" t="n">
-        <v>74.64</v>
+        <v>42.19</v>
       </c>
       <c r="AH12" t="n">
-        <v>75.95</v>
+        <v>46.89</v>
       </c>
       <c r="AI12" t="n">
-        <v>77.25</v>
+        <v>51.59</v>
       </c>
       <c r="AJ12" t="n">
-        <v>78.56</v>
+        <v>56.28</v>
       </c>
     </row>
     <row r="13">
@@ -2114,88 +2114,88 @@
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>1241.42</v>
+        <v>1212.64</v>
       </c>
       <c r="J13" t="n">
-        <v>1279.49</v>
+        <v>1244.28</v>
       </c>
       <c r="K13" t="n">
-        <v>1317.71</v>
+        <v>1275.93</v>
       </c>
       <c r="L13" t="n">
-        <v>1355.13</v>
+        <v>1340.26</v>
       </c>
       <c r="M13" t="n">
-        <v>1392.55</v>
+        <v>1404.59</v>
       </c>
       <c r="N13" t="n">
-        <v>1429.98</v>
+        <v>1468.93</v>
       </c>
       <c r="O13" t="n">
-        <v>1467.4</v>
+        <v>1533.26</v>
       </c>
       <c r="P13" t="n">
-        <v>1504.82</v>
+        <v>1597.59</v>
       </c>
       <c r="Q13" t="n">
-        <v>1542.24</v>
+        <v>1668.19</v>
       </c>
       <c r="R13" t="n">
-        <v>1579.67</v>
+        <v>1738.78</v>
       </c>
       <c r="S13" t="n">
-        <v>1617.09</v>
+        <v>1809.38</v>
       </c>
       <c r="T13" t="n">
-        <v>1654.51</v>
+        <v>1879.97</v>
       </c>
       <c r="U13" t="n">
-        <v>1691.93</v>
+        <v>1950.57</v>
       </c>
       <c r="V13" t="n">
-        <v>1729.36</v>
+        <v>2027.16</v>
       </c>
       <c r="W13" t="n">
-        <v>1766.78</v>
+        <v>2103.75</v>
       </c>
       <c r="X13" t="n">
-        <v>1804.2</v>
+        <v>2180.34</v>
       </c>
       <c r="Y13" t="n">
-        <v>1841.62</v>
+        <v>2256.94</v>
       </c>
       <c r="Z13" t="n">
-        <v>1879.05</v>
+        <v>2333.53</v>
       </c>
       <c r="AA13" t="n">
-        <v>1916.47</v>
+        <v>2418.53</v>
       </c>
       <c r="AB13" t="n">
-        <v>1953.89</v>
+        <v>2503.54</v>
       </c>
       <c r="AC13" t="n">
-        <v>1991.31</v>
+        <v>2588.55</v>
       </c>
       <c r="AD13" t="n">
-        <v>2028.74</v>
+        <v>2673.56</v>
       </c>
       <c r="AE13" t="n">
-        <v>2066.16</v>
+        <v>2758.57</v>
       </c>
       <c r="AF13" t="n">
-        <v>2103.58</v>
+        <v>2853.23</v>
       </c>
       <c r="AG13" t="n">
-        <v>2141</v>
+        <v>2947.89</v>
       </c>
       <c r="AH13" t="n">
-        <v>2178.43</v>
+        <v>3042.55</v>
       </c>
       <c r="AI13" t="n">
-        <v>2215.85</v>
+        <v>3137.21</v>
       </c>
       <c r="AJ13" t="n">
-        <v>2253.27</v>
+        <v>3231.87</v>
       </c>
     </row>
     <row r="14">
@@ -2238,88 +2238,88 @@
         <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>20.33</v>
+        <v>16.52</v>
       </c>
       <c r="J14" t="n">
-        <v>21.29</v>
+        <v>16.52</v>
       </c>
       <c r="K14" t="n">
-        <v>22.45</v>
+        <v>16.52</v>
       </c>
       <c r="L14" t="n">
-        <v>23.24</v>
+        <v>16.52</v>
       </c>
       <c r="M14" t="n">
-        <v>24.03</v>
+        <v>16.52</v>
       </c>
       <c r="N14" t="n">
-        <v>24.83</v>
+        <v>16.52</v>
       </c>
       <c r="O14" t="n">
-        <v>25.62</v>
+        <v>16.52</v>
       </c>
       <c r="P14" t="n">
-        <v>26.42</v>
+        <v>16.52</v>
       </c>
       <c r="Q14" t="n">
-        <v>27.21</v>
+        <v>16.52</v>
       </c>
       <c r="R14" t="n">
-        <v>28.01</v>
+        <v>16.52</v>
       </c>
       <c r="S14" t="n">
-        <v>28.8</v>
+        <v>16.52</v>
       </c>
       <c r="T14" t="n">
-        <v>29.6</v>
+        <v>16.52</v>
       </c>
       <c r="U14" t="n">
-        <v>30.39</v>
+        <v>16.52</v>
       </c>
       <c r="V14" t="n">
-        <v>31.19</v>
+        <v>16.52</v>
       </c>
       <c r="W14" t="n">
-        <v>31.98</v>
+        <v>16.52</v>
       </c>
       <c r="X14" t="n">
-        <v>32.77</v>
+        <v>16.52</v>
       </c>
       <c r="Y14" t="n">
-        <v>33.57</v>
+        <v>16.52</v>
       </c>
       <c r="Z14" t="n">
-        <v>34.36</v>
+        <v>16.52</v>
       </c>
       <c r="AA14" t="n">
-        <v>35.16</v>
+        <v>16.66</v>
       </c>
       <c r="AB14" t="n">
-        <v>35.95</v>
+        <v>16.8</v>
       </c>
       <c r="AC14" t="n">
-        <v>36.75</v>
+        <v>16.94</v>
       </c>
       <c r="AD14" t="n">
-        <v>37.54</v>
+        <v>17.08</v>
       </c>
       <c r="AE14" t="n">
-        <v>38.34</v>
+        <v>17.22</v>
       </c>
       <c r="AF14" t="n">
-        <v>39.13</v>
+        <v>20.52</v>
       </c>
       <c r="AG14" t="n">
-        <v>39.93</v>
+        <v>23.82</v>
       </c>
       <c r="AH14" t="n">
-        <v>40.72</v>
+        <v>27.12</v>
       </c>
       <c r="AI14" t="n">
-        <v>41.51</v>
+        <v>30.41</v>
       </c>
       <c r="AJ14" t="n">
-        <v>42.31</v>
+        <v>33.71</v>
       </c>
     </row>
     <row r="15">
@@ -2362,88 +2362,88 @@
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>51.79</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="J15" t="n">
-        <v>52.92</v>
+        <v>75.26000000000001</v>
       </c>
       <c r="K15" t="n">
-        <v>56.17</v>
+        <v>79.62</v>
       </c>
       <c r="L15" t="n">
-        <v>58.72</v>
+        <v>84.13</v>
       </c>
       <c r="M15" t="n">
-        <v>61.26</v>
+        <v>88.63</v>
       </c>
       <c r="N15" t="n">
-        <v>63.81</v>
+        <v>93.14</v>
       </c>
       <c r="O15" t="n">
-        <v>66.36</v>
+        <v>97.64</v>
       </c>
       <c r="P15" t="n">
-        <v>68.91</v>
+        <v>102.15</v>
       </c>
       <c r="Q15" t="n">
-        <v>71.45</v>
+        <v>106.85</v>
       </c>
       <c r="R15" t="n">
-        <v>74</v>
+        <v>111.55</v>
       </c>
       <c r="S15" t="n">
-        <v>76.55</v>
+        <v>116.26</v>
       </c>
       <c r="T15" t="n">
-        <v>79.09999999999999</v>
+        <v>120.96</v>
       </c>
       <c r="U15" t="n">
-        <v>81.64</v>
+        <v>125.66</v>
       </c>
       <c r="V15" t="n">
-        <v>84.19</v>
+        <v>130.6</v>
       </c>
       <c r="W15" t="n">
-        <v>86.73999999999999</v>
+        <v>135.55</v>
       </c>
       <c r="X15" t="n">
-        <v>89.29000000000001</v>
+        <v>140.49</v>
       </c>
       <c r="Y15" t="n">
-        <v>91.84</v>
+        <v>145.43</v>
       </c>
       <c r="Z15" t="n">
-        <v>94.38</v>
+        <v>150.37</v>
       </c>
       <c r="AA15" t="n">
-        <v>96.93000000000001</v>
+        <v>155.7</v>
       </c>
       <c r="AB15" t="n">
-        <v>99.48</v>
+        <v>161.04</v>
       </c>
       <c r="AC15" t="n">
-        <v>102.03</v>
+        <v>166.37</v>
       </c>
       <c r="AD15" t="n">
-        <v>104.57</v>
+        <v>171.7</v>
       </c>
       <c r="AE15" t="n">
-        <v>107.12</v>
+        <v>177.03</v>
       </c>
       <c r="AF15" t="n">
-        <v>109.67</v>
+        <v>182.55</v>
       </c>
       <c r="AG15" t="n">
-        <v>112.22</v>
+        <v>188.07</v>
       </c>
       <c r="AH15" t="n">
-        <v>114.76</v>
+        <v>193.58</v>
       </c>
       <c r="AI15" t="n">
-        <v>117.31</v>
+        <v>199.1</v>
       </c>
       <c r="AJ15" t="n">
-        <v>119.86</v>
+        <v>204.62</v>
       </c>
     </row>
     <row r="16">
@@ -2486,88 +2486,88 @@
         <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>223.04</v>
+        <v>257.51</v>
       </c>
       <c r="J16" t="n">
-        <v>233.01</v>
+        <v>266.64</v>
       </c>
       <c r="K16" t="n">
-        <v>242.56</v>
+        <v>275.78</v>
       </c>
       <c r="L16" t="n">
-        <v>252.12</v>
+        <v>284.8</v>
       </c>
       <c r="M16" t="n">
-        <v>261.68</v>
+        <v>293.82</v>
       </c>
       <c r="N16" t="n">
-        <v>271.25</v>
+        <v>302.84</v>
       </c>
       <c r="O16" t="n">
-        <v>280.81</v>
+        <v>311.86</v>
       </c>
       <c r="P16" t="n">
-        <v>290.37</v>
+        <v>320.88</v>
       </c>
       <c r="Q16" t="n">
-        <v>299.94</v>
+        <v>330</v>
       </c>
       <c r="R16" t="n">
-        <v>309.5</v>
+        <v>339.12</v>
       </c>
       <c r="S16" t="n">
-        <v>319.07</v>
+        <v>348.24</v>
       </c>
       <c r="T16" t="n">
-        <v>328.63</v>
+        <v>357.36</v>
       </c>
       <c r="U16" t="n">
-        <v>338.19</v>
+        <v>366.48</v>
       </c>
       <c r="V16" t="n">
-        <v>347.76</v>
+        <v>376.05</v>
       </c>
       <c r="W16" t="n">
-        <v>357.32</v>
+        <v>385.63</v>
       </c>
       <c r="X16" t="n">
-        <v>366.88</v>
+        <v>395.21</v>
       </c>
       <c r="Y16" t="n">
-        <v>376.45</v>
+        <v>404.78</v>
       </c>
       <c r="Z16" t="n">
-        <v>386.01</v>
+        <v>414.36</v>
       </c>
       <c r="AA16" t="n">
-        <v>395.57</v>
+        <v>424.36</v>
       </c>
       <c r="AB16" t="n">
-        <v>405.14</v>
+        <v>434.36</v>
       </c>
       <c r="AC16" t="n">
-        <v>414.7</v>
+        <v>444.37</v>
       </c>
       <c r="AD16" t="n">
-        <v>424.26</v>
+        <v>454.37</v>
       </c>
       <c r="AE16" t="n">
-        <v>433.83</v>
+        <v>464.37</v>
       </c>
       <c r="AF16" t="n">
-        <v>443.39</v>
+        <v>474.65</v>
       </c>
       <c r="AG16" t="n">
-        <v>452.96</v>
+        <v>484.93</v>
       </c>
       <c r="AH16" t="n">
-        <v>462.52</v>
+        <v>495.2</v>
       </c>
       <c r="AI16" t="n">
-        <v>472.08</v>
+        <v>505.48</v>
       </c>
       <c r="AJ16" t="n">
-        <v>481.65</v>
+        <v>515.76</v>
       </c>
     </row>
     <row r="17">
@@ -2610,88 +2610,88 @@
         <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>81.55</v>
+        <v>52.63</v>
       </c>
       <c r="J17" t="n">
-        <v>145.53</v>
+        <v>52.63</v>
       </c>
       <c r="K17" t="n">
-        <v>128.87</v>
+        <v>52.63</v>
       </c>
       <c r="L17" t="n">
-        <v>141.05</v>
+        <v>52.63</v>
       </c>
       <c r="M17" t="n">
-        <v>153.23</v>
+        <v>52.63</v>
       </c>
       <c r="N17" t="n">
-        <v>165.41</v>
+        <v>52.63</v>
       </c>
       <c r="O17" t="n">
-        <v>177.6</v>
+        <v>52.63</v>
       </c>
       <c r="P17" t="n">
-        <v>189.78</v>
+        <v>52.63</v>
       </c>
       <c r="Q17" t="n">
-        <v>201.96</v>
+        <v>52.63</v>
       </c>
       <c r="R17" t="n">
-        <v>214.14</v>
+        <v>52.63</v>
       </c>
       <c r="S17" t="n">
-        <v>226.33</v>
+        <v>52.63</v>
       </c>
       <c r="T17" t="n">
-        <v>238.51</v>
+        <v>52.63</v>
       </c>
       <c r="U17" t="n">
-        <v>250.69</v>
+        <v>52.63</v>
       </c>
       <c r="V17" t="n">
-        <v>262.87</v>
+        <v>54.53</v>
       </c>
       <c r="W17" t="n">
-        <v>275.06</v>
+        <v>56.44</v>
       </c>
       <c r="X17" t="n">
-        <v>287.24</v>
+        <v>58.34</v>
       </c>
       <c r="Y17" t="n">
-        <v>299.42</v>
+        <v>60.24</v>
       </c>
       <c r="Z17" t="n">
-        <v>311.6</v>
+        <v>62.14</v>
       </c>
       <c r="AA17" t="n">
-        <v>323.79</v>
+        <v>64.7</v>
       </c>
       <c r="AB17" t="n">
-        <v>335.97</v>
+        <v>67.26000000000001</v>
       </c>
       <c r="AC17" t="n">
-        <v>348.15</v>
+        <v>69.81999999999999</v>
       </c>
       <c r="AD17" t="n">
-        <v>360.34</v>
+        <v>72.38</v>
       </c>
       <c r="AE17" t="n">
-        <v>372.52</v>
+        <v>74.94</v>
       </c>
       <c r="AF17" t="n">
-        <v>384.7</v>
+        <v>77.86</v>
       </c>
       <c r="AG17" t="n">
-        <v>396.88</v>
+        <v>80.78</v>
       </c>
       <c r="AH17" t="n">
-        <v>409.07</v>
+        <v>83.7</v>
       </c>
       <c r="AI17" t="n">
-        <v>421.25</v>
+        <v>86.62</v>
       </c>
       <c r="AJ17" t="n">
-        <v>433.43</v>
+        <v>89.54000000000001</v>
       </c>
     </row>
     <row r="18">
@@ -2734,88 +2734,88 @@
         <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>27.94</v>
+        <v>24.8</v>
       </c>
       <c r="J18" t="n">
-        <v>29.86</v>
+        <v>24.8</v>
       </c>
       <c r="K18" t="n">
-        <v>32.04</v>
+        <v>24.8</v>
       </c>
       <c r="L18" t="n">
-        <v>32.72</v>
+        <v>24.8</v>
       </c>
       <c r="M18" t="n">
-        <v>33.4</v>
+        <v>24.8</v>
       </c>
       <c r="N18" t="n">
-        <v>34.08</v>
+        <v>24.8</v>
       </c>
       <c r="O18" t="n">
-        <v>34.75</v>
+        <v>24.8</v>
       </c>
       <c r="P18" t="n">
-        <v>35.43</v>
+        <v>24.8</v>
       </c>
       <c r="Q18" t="n">
-        <v>36.11</v>
+        <v>24.8</v>
       </c>
       <c r="R18" t="n">
-        <v>36.79</v>
+        <v>24.8</v>
       </c>
       <c r="S18" t="n">
-        <v>37.47</v>
+        <v>24.8</v>
       </c>
       <c r="T18" t="n">
-        <v>38.14</v>
+        <v>24.8</v>
       </c>
       <c r="U18" t="n">
-        <v>38.82</v>
+        <v>24.8</v>
       </c>
       <c r="V18" t="n">
-        <v>39.5</v>
+        <v>24.86</v>
       </c>
       <c r="W18" t="n">
-        <v>40.18</v>
+        <v>24.92</v>
       </c>
       <c r="X18" t="n">
-        <v>40.86</v>
+        <v>24.98</v>
       </c>
       <c r="Y18" t="n">
-        <v>41.53</v>
+        <v>25.05</v>
       </c>
       <c r="Z18" t="n">
-        <v>42.21</v>
+        <v>25.11</v>
       </c>
       <c r="AA18" t="n">
-        <v>42.89</v>
+        <v>27.13</v>
       </c>
       <c r="AB18" t="n">
-        <v>43.57</v>
+        <v>29.15</v>
       </c>
       <c r="AC18" t="n">
-        <v>44.24</v>
+        <v>31.17</v>
       </c>
       <c r="AD18" t="n">
-        <v>44.92</v>
+        <v>33.19</v>
       </c>
       <c r="AE18" t="n">
-        <v>45.6</v>
+        <v>35.22</v>
       </c>
       <c r="AF18" t="n">
-        <v>46.28</v>
+        <v>37.46</v>
       </c>
       <c r="AG18" t="n">
-        <v>46.96</v>
+        <v>39.71</v>
       </c>
       <c r="AH18" t="n">
-        <v>47.63</v>
+        <v>41.95</v>
       </c>
       <c r="AI18" t="n">
-        <v>48.31</v>
+        <v>44.2</v>
       </c>
       <c r="AJ18" t="n">
-        <v>48.99</v>
+        <v>46.44</v>
       </c>
     </row>
     <row r="19">
@@ -2858,212 +2858,88 @@
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>50.51</v>
+        <v>44.75</v>
       </c>
       <c r="J19" t="n">
-        <v>40.18</v>
+        <v>44.75</v>
       </c>
       <c r="K19" t="n">
-        <v>44.5</v>
+        <v>44.75</v>
       </c>
       <c r="L19" t="n">
-        <v>45.59</v>
+        <v>44.75</v>
       </c>
       <c r="M19" t="n">
-        <v>46.68</v>
+        <v>44.75</v>
       </c>
       <c r="N19" t="n">
-        <v>47.78</v>
+        <v>44.75</v>
       </c>
       <c r="O19" t="n">
-        <v>48.87</v>
+        <v>44.75</v>
       </c>
       <c r="P19" t="n">
-        <v>49.97</v>
+        <v>44.75</v>
       </c>
       <c r="Q19" t="n">
-        <v>51.06</v>
+        <v>45.2</v>
       </c>
       <c r="R19" t="n">
-        <v>52.15</v>
+        <v>45.66</v>
       </c>
       <c r="S19" t="n">
-        <v>53.25</v>
+        <v>46.12</v>
       </c>
       <c r="T19" t="n">
-        <v>54.34</v>
+        <v>46.57</v>
       </c>
       <c r="U19" t="n">
-        <v>55.44</v>
+        <v>47.03</v>
       </c>
       <c r="V19" t="n">
-        <v>56.53</v>
+        <v>47.83</v>
       </c>
       <c r="W19" t="n">
-        <v>57.62</v>
+        <v>48.62</v>
       </c>
       <c r="X19" t="n">
-        <v>58.72</v>
+        <v>49.42</v>
       </c>
       <c r="Y19" t="n">
-        <v>59.81</v>
+        <v>50.22</v>
       </c>
       <c r="Z19" t="n">
-        <v>60.91</v>
+        <v>51.02</v>
       </c>
       <c r="AA19" t="n">
-        <v>62</v>
+        <v>51.86</v>
       </c>
       <c r="AB19" t="n">
-        <v>63.09</v>
+        <v>52.69</v>
       </c>
       <c r="AC19" t="n">
-        <v>64.19</v>
+        <v>53.53</v>
       </c>
       <c r="AD19" t="n">
-        <v>65.28</v>
+        <v>54.36</v>
       </c>
       <c r="AE19" t="n">
-        <v>66.38</v>
+        <v>55.2</v>
       </c>
       <c r="AF19" t="n">
-        <v>67.47</v>
+        <v>56.05</v>
       </c>
       <c r="AG19" t="n">
-        <v>68.56</v>
+        <v>56.9</v>
       </c>
       <c r="AH19" t="n">
-        <v>69.66</v>
+        <v>57.75</v>
       </c>
       <c r="AI19" t="n">
-        <v>70.75</v>
+        <v>58.59</v>
       </c>
       <c r="AJ19" t="n">
-        <v>71.84999999999999</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Demand</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>ELCHTIXX03</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Output demand of dispatch-ready in Haiti</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>not needed</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>not needed</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>not needed</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>User defined</t>
-        </is>
-      </c>
-      <c r="H20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" t="n">
-        <v>3.13</v>
-      </c>
-      <c r="J20" t="n">
-        <v>3.23</v>
-      </c>
-      <c r="K20" t="n">
-        <v>3.33</v>
-      </c>
-      <c r="L20" t="n">
-        <v>3.43</v>
-      </c>
-      <c r="M20" t="n">
-        <v>3.53</v>
-      </c>
-      <c r="N20" t="n">
-        <v>3.63</v>
-      </c>
-      <c r="O20" t="n">
-        <v>3.73</v>
-      </c>
-      <c r="P20" t="n">
-        <v>3.83</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>3.93</v>
-      </c>
-      <c r="R20" t="n">
-        <v>4.03</v>
-      </c>
-      <c r="S20" t="n">
-        <v>4.13</v>
-      </c>
-      <c r="T20" t="n">
-        <v>4.23</v>
-      </c>
-      <c r="U20" t="n">
-        <v>4.33</v>
-      </c>
-      <c r="V20" t="n">
-        <v>4.43</v>
-      </c>
-      <c r="W20" t="n">
-        <v>4.53</v>
-      </c>
-      <c r="X20" t="n">
-        <v>4.63</v>
-      </c>
-      <c r="Y20" t="n">
-        <v>4.73</v>
-      </c>
-      <c r="Z20" t="n">
-        <v>4.83</v>
-      </c>
-      <c r="AA20" t="n">
-        <v>4.93</v>
-      </c>
-      <c r="AB20" t="n">
-        <v>5.03</v>
-      </c>
-      <c r="AC20" t="n">
-        <v>5.13</v>
-      </c>
-      <c r="AD20" t="n">
-        <v>5.23</v>
-      </c>
-      <c r="AE20" t="n">
-        <v>5.34</v>
-      </c>
-      <c r="AF20" t="n">
-        <v>5.44</v>
-      </c>
-      <c r="AG20" t="n">
-        <v>5.54</v>
-      </c>
-      <c r="AH20" t="n">
-        <v>5.64</v>
-      </c>
-      <c r="AI20" t="n">
-        <v>5.74</v>
-      </c>
-      <c r="AJ20" t="n">
-        <v>5.84</v>
+        <v>59.44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update demand with projection of NZE scenario from WEO
</commit_message>
<xml_diff>
--- a/t1_confection/A1_Outputs/A1_Outputs_BAU/A-O_Demand.xlsx
+++ b/t1_confection/A1_Outputs/A1_Outputs_BAU/A-O_Demand.xlsx
@@ -750,88 +750,88 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>524.49</v>
+        <v>558.829268292683</v>
       </c>
       <c r="J2" t="n">
-        <v>529.1</v>
+        <v>572.8</v>
       </c>
       <c r="K2" t="n">
-        <v>533.72</v>
+        <v>595.66</v>
       </c>
       <c r="L2" t="n">
-        <v>538.33</v>
+        <v>619.25</v>
       </c>
       <c r="M2" t="n">
-        <v>542.95</v>
+        <v>643.61</v>
       </c>
       <c r="N2" t="n">
-        <v>547.5599999999999</v>
+        <v>668.75</v>
       </c>
       <c r="O2" t="n">
-        <v>552.1799999999999</v>
+        <v>694.6900000000001</v>
       </c>
       <c r="P2" t="n">
-        <v>556.79</v>
+        <v>721.46</v>
       </c>
       <c r="Q2" t="n">
-        <v>561.41</v>
+        <v>749.09</v>
       </c>
       <c r="R2" t="n">
-        <v>566.03</v>
+        <v>777.59</v>
       </c>
       <c r="S2" t="n">
-        <v>570.64</v>
+        <v>806.99</v>
       </c>
       <c r="T2" t="n">
-        <v>575.26</v>
+        <v>837.33</v>
       </c>
       <c r="U2" t="n">
-        <v>579.87</v>
+        <v>868.62</v>
       </c>
       <c r="V2" t="n">
-        <v>584.49</v>
+        <v>907.0599999999999</v>
       </c>
       <c r="W2" t="n">
-        <v>589.1</v>
+        <v>946.55</v>
       </c>
       <c r="X2" t="n">
-        <v>593.72</v>
+        <v>987.13</v>
       </c>
       <c r="Y2" t="n">
-        <v>598.33</v>
+        <v>1028.81</v>
       </c>
       <c r="Z2" t="n">
-        <v>602.95</v>
+        <v>1071.62</v>
       </c>
       <c r="AA2" t="n">
-        <v>607.5599999999999</v>
+        <v>1115.59</v>
       </c>
       <c r="AB2" t="n">
-        <v>612.1799999999999</v>
+        <v>1160.75</v>
       </c>
       <c r="AC2" t="n">
-        <v>616.8</v>
+        <v>1207.12</v>
       </c>
       <c r="AD2" t="n">
-        <v>621.41</v>
+        <v>1254.73</v>
       </c>
       <c r="AE2" t="n">
-        <v>626.03</v>
+        <v>1303.61</v>
       </c>
       <c r="AF2" t="n">
-        <v>630.64</v>
+        <v>1353.79</v>
       </c>
       <c r="AG2" t="n">
-        <v>635.26</v>
+        <v>1405.3</v>
       </c>
       <c r="AH2" t="n">
-        <v>639.87</v>
+        <v>1458.17</v>
       </c>
       <c r="AI2" t="n">
-        <v>644.49</v>
+        <v>1512.43</v>
       </c>
       <c r="AJ2" t="n">
-        <v>649.1</v>
+        <v>1568.11</v>
       </c>
     </row>
     <row r="3">
@@ -874,88 +874,88 @@
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>42.81</v>
+        <v>41.39512195121952</v>
       </c>
       <c r="J3" t="n">
-        <v>45.54</v>
+        <v>42.43</v>
       </c>
       <c r="K3" t="n">
-        <v>48.27</v>
+        <v>44.71</v>
       </c>
       <c r="L3" t="n">
-        <v>51.01</v>
+        <v>47.09</v>
       </c>
       <c r="M3" t="n">
-        <v>53.74</v>
+        <v>49.59</v>
       </c>
       <c r="N3" t="n">
-        <v>56.47</v>
+        <v>52.21</v>
       </c>
       <c r="O3" t="n">
-        <v>59.2</v>
+        <v>54.95</v>
       </c>
       <c r="P3" t="n">
-        <v>61.93</v>
+        <v>57.82</v>
       </c>
       <c r="Q3" t="n">
-        <v>64.66</v>
+        <v>60.82</v>
       </c>
       <c r="R3" t="n">
-        <v>67.39</v>
+        <v>63.97</v>
       </c>
       <c r="S3" t="n">
-        <v>70.13</v>
+        <v>67.27</v>
       </c>
       <c r="T3" t="n">
-        <v>72.86</v>
+        <v>70.72</v>
       </c>
       <c r="U3" t="n">
-        <v>75.59</v>
+        <v>74.33</v>
       </c>
       <c r="V3" t="n">
-        <v>78.31999999999999</v>
+        <v>78.44</v>
       </c>
       <c r="W3" t="n">
-        <v>81.05</v>
+        <v>82.73</v>
       </c>
       <c r="X3" t="n">
-        <v>83.78</v>
+        <v>87.19</v>
       </c>
       <c r="Y3" t="n">
-        <v>86.51000000000001</v>
+        <v>91.84</v>
       </c>
       <c r="Z3" t="n">
-        <v>89.25</v>
+        <v>96.67</v>
       </c>
       <c r="AA3" t="n">
-        <v>91.98</v>
+        <v>101.71</v>
       </c>
       <c r="AB3" t="n">
-        <v>94.70999999999999</v>
+        <v>106.95</v>
       </c>
       <c r="AC3" t="n">
-        <v>97.44</v>
+        <v>112.4</v>
       </c>
       <c r="AD3" t="n">
-        <v>100.17</v>
+        <v>118.08</v>
       </c>
       <c r="AE3" t="n">
-        <v>102.9</v>
+        <v>123.98</v>
       </c>
       <c r="AF3" t="n">
-        <v>105.63</v>
+        <v>130.12</v>
       </c>
       <c r="AG3" t="n">
-        <v>108.37</v>
+        <v>136.5</v>
       </c>
       <c r="AH3" t="n">
-        <v>111.1</v>
+        <v>143.14</v>
       </c>
       <c r="AI3" t="n">
-        <v>113.83</v>
+        <v>150.05</v>
       </c>
       <c r="AJ3" t="n">
-        <v>116.56</v>
+        <v>157.22</v>
       </c>
     </row>
     <row r="4">
@@ -998,88 +998,88 @@
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>2599.63</v>
+        <v>2237.268292682927</v>
       </c>
       <c r="J4" t="n">
-        <v>2656.56</v>
+        <v>2293.2</v>
       </c>
       <c r="K4" t="n">
-        <v>2713.49</v>
+        <v>2374.59</v>
       </c>
       <c r="L4" t="n">
-        <v>2770.42</v>
+        <v>2458.36</v>
       </c>
       <c r="M4" t="n">
-        <v>2827.36</v>
+        <v>2544.56</v>
       </c>
       <c r="N4" t="n">
-        <v>2884.29</v>
+        <v>2633.26</v>
       </c>
       <c r="O4" t="n">
-        <v>2941.22</v>
+        <v>2724.53</v>
       </c>
       <c r="P4" t="n">
-        <v>2998.15</v>
+        <v>2818.44</v>
       </c>
       <c r="Q4" t="n">
-        <v>3055.08</v>
+        <v>2915.05</v>
       </c>
       <c r="R4" t="n">
-        <v>3112.02</v>
+        <v>3014.44</v>
       </c>
       <c r="S4" t="n">
-        <v>3168.95</v>
+        <v>3116.67</v>
       </c>
       <c r="T4" t="n">
-        <v>3225.88</v>
+        <v>3221.84</v>
       </c>
       <c r="U4" t="n">
-        <v>3282.81</v>
+        <v>3330</v>
       </c>
       <c r="V4" t="n">
-        <v>3339.74</v>
+        <v>3458.25</v>
       </c>
       <c r="W4" t="n">
-        <v>3396.67</v>
+        <v>3589.65</v>
       </c>
       <c r="X4" t="n">
-        <v>3453.61</v>
+        <v>3724.26</v>
       </c>
       <c r="Y4" t="n">
-        <v>3510.54</v>
+        <v>3862.15</v>
       </c>
       <c r="Z4" t="n">
-        <v>3567.47</v>
+        <v>4003.39</v>
       </c>
       <c r="AA4" t="n">
-        <v>3624.4</v>
+        <v>4148.04</v>
       </c>
       <c r="AB4" t="n">
-        <v>3681.33</v>
+        <v>4296.19</v>
       </c>
       <c r="AC4" t="n">
-        <v>3738.27</v>
+        <v>4447.89</v>
       </c>
       <c r="AD4" t="n">
-        <v>3795.2</v>
+        <v>4603.23</v>
       </c>
       <c r="AE4" t="n">
-        <v>3852.13</v>
+        <v>4762.29</v>
       </c>
       <c r="AF4" t="n">
-        <v>3909.06</v>
+        <v>4925.13</v>
       </c>
       <c r="AG4" t="n">
-        <v>3965.99</v>
+        <v>5091.84</v>
       </c>
       <c r="AH4" t="n">
-        <v>4022.93</v>
+        <v>5262.5</v>
       </c>
       <c r="AI4" t="n">
-        <v>4079.86</v>
+        <v>5437.2</v>
       </c>
       <c r="AJ4" t="n">
-        <v>4136.79</v>
+        <v>5616</v>
       </c>
     </row>
     <row r="5">
@@ -1122,88 +1122,88 @@
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>3.87</v>
+        <v>4.13658536585366</v>
       </c>
       <c r="J5" t="n">
-        <v>4.08</v>
+        <v>4.24</v>
       </c>
       <c r="K5" t="n">
-        <v>4.29</v>
+        <v>4.37</v>
       </c>
       <c r="L5" t="n">
         <v>4.49</v>
       </c>
       <c r="M5" t="n">
-        <v>4.7</v>
+        <v>4.62</v>
       </c>
       <c r="N5" t="n">
-        <v>4.91</v>
+        <v>4.75</v>
       </c>
       <c r="O5" t="n">
-        <v>5.12</v>
+        <v>4.89</v>
       </c>
       <c r="P5" t="n">
-        <v>5.32</v>
+        <v>5.02</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.53</v>
+        <v>5.16</v>
       </c>
       <c r="R5" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="S5" t="n">
+        <v>5.45</v>
+      </c>
+      <c r="T5" t="n">
+        <v>5.59</v>
+      </c>
+      <c r="U5" t="n">
         <v>5.74</v>
       </c>
-      <c r="S5" t="n">
+      <c r="V5" t="n">
         <v>5.94</v>
       </c>
-      <c r="T5" t="n">
-        <v>6.15</v>
-      </c>
-      <c r="U5" t="n">
-        <v>6.36</v>
-      </c>
-      <c r="V5" t="n">
-        <v>6.56</v>
-      </c>
       <c r="W5" t="n">
-        <v>6.77</v>
+        <v>6.14</v>
       </c>
       <c r="X5" t="n">
-        <v>6.98</v>
+        <v>6.34</v>
       </c>
       <c r="Y5" t="n">
-        <v>7.18</v>
+        <v>6.54</v>
       </c>
       <c r="Z5" t="n">
-        <v>7.39</v>
+        <v>6.74</v>
       </c>
       <c r="AA5" t="n">
-        <v>7.6</v>
+        <v>6.95</v>
       </c>
       <c r="AB5" t="n">
-        <v>7.8</v>
+        <v>7.16</v>
       </c>
       <c r="AC5" t="n">
-        <v>8.01</v>
+        <v>7.38</v>
       </c>
       <c r="AD5" t="n">
-        <v>8.220000000000001</v>
+        <v>7.59</v>
       </c>
       <c r="AE5" t="n">
-        <v>8.43</v>
+        <v>7.81</v>
       </c>
       <c r="AF5" t="n">
-        <v>8.630000000000001</v>
+        <v>8.029999999999999</v>
       </c>
       <c r="AG5" t="n">
-        <v>8.84</v>
+        <v>8.25</v>
       </c>
       <c r="AH5" t="n">
-        <v>9.050000000000001</v>
+        <v>8.48</v>
       </c>
       <c r="AI5" t="n">
-        <v>9.25</v>
+        <v>8.710000000000001</v>
       </c>
       <c r="AJ5" t="n">
-        <v>9.460000000000001</v>
+        <v>8.94</v>
       </c>
     </row>
     <row r="6">
@@ -1246,88 +1246,88 @@
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>302.26</v>
+        <v>339.4341463414635</v>
       </c>
       <c r="J6" t="n">
-        <v>313.41</v>
+        <v>347.92</v>
       </c>
       <c r="K6" t="n">
-        <v>324.56</v>
+        <v>359.86</v>
       </c>
       <c r="L6" t="n">
-        <v>335.71</v>
+        <v>372.1</v>
       </c>
       <c r="M6" t="n">
-        <v>346.87</v>
+        <v>384.66</v>
       </c>
       <c r="N6" t="n">
-        <v>358.02</v>
+        <v>397.53</v>
       </c>
       <c r="O6" t="n">
-        <v>369.17</v>
+        <v>410.73</v>
       </c>
       <c r="P6" t="n">
-        <v>380.33</v>
+        <v>424.27</v>
       </c>
       <c r="Q6" t="n">
-        <v>391.48</v>
+        <v>438.14</v>
       </c>
       <c r="R6" t="n">
-        <v>402.63</v>
+        <v>452.37</v>
       </c>
       <c r="S6" t="n">
-        <v>413.79</v>
+        <v>466.95</v>
       </c>
       <c r="T6" t="n">
-        <v>424.94</v>
+        <v>481.9</v>
       </c>
       <c r="U6" t="n">
-        <v>436.09</v>
+        <v>497.22</v>
       </c>
       <c r="V6" t="n">
-        <v>447.25</v>
+        <v>516.3099999999999</v>
       </c>
       <c r="W6" t="n">
-        <v>458.4</v>
+        <v>535.77</v>
       </c>
       <c r="X6" t="n">
-        <v>469.55</v>
+        <v>555.6</v>
       </c>
       <c r="Y6" t="n">
-        <v>480.71</v>
+        <v>575.8200000000001</v>
       </c>
       <c r="Z6" t="n">
-        <v>491.86</v>
+        <v>596.42</v>
       </c>
       <c r="AA6" t="n">
-        <v>503.01</v>
+        <v>617.41</v>
       </c>
       <c r="AB6" t="n">
-        <v>514.17</v>
+        <v>638.8</v>
       </c>
       <c r="AC6" t="n">
-        <v>525.3200000000001</v>
+        <v>660.6</v>
       </c>
       <c r="AD6" t="n">
-        <v>536.47</v>
+        <v>682.8</v>
       </c>
       <c r="AE6" t="n">
-        <v>547.63</v>
+        <v>705.4299999999999</v>
       </c>
       <c r="AF6" t="n">
-        <v>558.78</v>
+        <v>728.48</v>
       </c>
       <c r="AG6" t="n">
-        <v>569.9299999999999</v>
+        <v>751.95</v>
       </c>
       <c r="AH6" t="n">
-        <v>581.09</v>
+        <v>775.87</v>
       </c>
       <c r="AI6" t="n">
-        <v>592.24</v>
+        <v>800.23</v>
       </c>
       <c r="AJ6" t="n">
-        <v>603.39</v>
+        <v>825.04</v>
       </c>
     </row>
     <row r="7">
@@ -1370,88 +1370,88 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>288.23</v>
+        <v>310.4585365853659</v>
       </c>
       <c r="J7" t="n">
-        <v>294.17</v>
+        <v>318.22</v>
       </c>
       <c r="K7" t="n">
-        <v>300.1</v>
+        <v>334.51</v>
       </c>
       <c r="L7" t="n">
-        <v>306.04</v>
+        <v>351.54</v>
       </c>
       <c r="M7" t="n">
-        <v>311.98</v>
+        <v>369.33</v>
       </c>
       <c r="N7" t="n">
-        <v>317.92</v>
+        <v>387.92</v>
       </c>
       <c r="O7" t="n">
-        <v>323.85</v>
+        <v>407.35</v>
       </c>
       <c r="P7" t="n">
-        <v>329.79</v>
+        <v>427.64</v>
       </c>
       <c r="Q7" t="n">
-        <v>335.73</v>
+        <v>448.83</v>
       </c>
       <c r="R7" t="n">
-        <v>341.67</v>
+        <v>470.97</v>
       </c>
       <c r="S7" t="n">
-        <v>347.6</v>
+        <v>494.08</v>
       </c>
       <c r="T7" t="n">
-        <v>353.54</v>
+        <v>518.22</v>
       </c>
       <c r="U7" t="n">
-        <v>359.48</v>
+        <v>543.42</v>
       </c>
       <c r="V7" t="n">
-        <v>365.42</v>
+        <v>572.33</v>
       </c>
       <c r="W7" t="n">
-        <v>371.35</v>
+        <v>602.36</v>
       </c>
       <c r="X7" t="n">
-        <v>377.29</v>
+        <v>633.55</v>
       </c>
       <c r="Y7" t="n">
-        <v>383.23</v>
+        <v>665.95</v>
       </c>
       <c r="Z7" t="n">
-        <v>389.17</v>
+        <v>699.6</v>
       </c>
       <c r="AA7" t="n">
-        <v>395.1</v>
+        <v>734.53</v>
       </c>
       <c r="AB7" t="n">
-        <v>401.04</v>
+        <v>770.8</v>
       </c>
       <c r="AC7" t="n">
-        <v>406.98</v>
+        <v>808.45</v>
       </c>
       <c r="AD7" t="n">
-        <v>412.92</v>
+        <v>847.53</v>
       </c>
       <c r="AE7" t="n">
-        <v>418.85</v>
+        <v>888.08</v>
       </c>
       <c r="AF7" t="n">
-        <v>424.79</v>
+        <v>930.15</v>
       </c>
       <c r="AG7" t="n">
-        <v>430.73</v>
+        <v>973.8</v>
       </c>
       <c r="AH7" t="n">
-        <v>436.67</v>
+        <v>1019.08</v>
       </c>
       <c r="AI7" t="n">
-        <v>442.6</v>
+        <v>1066.04</v>
       </c>
       <c r="AJ7" t="n">
-        <v>448.54</v>
+        <v>1114.75</v>
       </c>
     </row>
     <row r="8">
@@ -1494,88 +1494,88 @@
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>44.28</v>
+        <v>49.67804878048781</v>
       </c>
       <c r="J8" t="n">
-        <v>45.83</v>
+        <v>50.92</v>
       </c>
       <c r="K8" t="n">
-        <v>47.38</v>
+        <v>53.26</v>
       </c>
       <c r="L8" t="n">
-        <v>48.93</v>
+        <v>55.69</v>
       </c>
       <c r="M8" t="n">
-        <v>50.48</v>
+        <v>58.22</v>
       </c>
       <c r="N8" t="n">
-        <v>52.03</v>
+        <v>60.85</v>
       </c>
       <c r="O8" t="n">
-        <v>53.58</v>
+        <v>63.58</v>
       </c>
       <c r="P8" t="n">
-        <v>55.13</v>
+        <v>66.42</v>
       </c>
       <c r="Q8" t="n">
-        <v>56.68</v>
+        <v>69.37</v>
       </c>
       <c r="R8" t="n">
-        <v>58.23</v>
+        <v>72.43000000000001</v>
       </c>
       <c r="S8" t="n">
-        <v>59.78</v>
+        <v>75.61</v>
       </c>
       <c r="T8" t="n">
-        <v>61.33</v>
+        <v>78.91</v>
       </c>
       <c r="U8" t="n">
-        <v>62.88</v>
+        <v>82.34</v>
       </c>
       <c r="V8" t="n">
-        <v>64.43000000000001</v>
+        <v>86.34999999999999</v>
       </c>
       <c r="W8" t="n">
-        <v>65.98</v>
+        <v>90.48999999999999</v>
       </c>
       <c r="X8" t="n">
-        <v>67.53</v>
+        <v>94.77</v>
       </c>
       <c r="Y8" t="n">
-        <v>69.08</v>
+        <v>99.19</v>
       </c>
       <c r="Z8" t="n">
-        <v>70.63</v>
+        <v>103.75</v>
       </c>
       <c r="AA8" t="n">
-        <v>72.18000000000001</v>
+        <v>108.47</v>
       </c>
       <c r="AB8" t="n">
-        <v>73.73</v>
+        <v>113.33</v>
       </c>
       <c r="AC8" t="n">
-        <v>75.28</v>
+        <v>118.36</v>
       </c>
       <c r="AD8" t="n">
-        <v>76.83</v>
+        <v>123.55</v>
       </c>
       <c r="AE8" t="n">
-        <v>78.38</v>
+        <v>128.91</v>
       </c>
       <c r="AF8" t="n">
-        <v>79.93000000000001</v>
+        <v>134.43</v>
       </c>
       <c r="AG8" t="n">
-        <v>81.48</v>
+        <v>140.14</v>
       </c>
       <c r="AH8" t="n">
-        <v>83.03</v>
+        <v>146.02</v>
       </c>
       <c r="AI8" t="n">
-        <v>84.58</v>
+        <v>152.1</v>
       </c>
       <c r="AJ8" t="n">
-        <v>86.13</v>
+        <v>158.37</v>
       </c>
     </row>
     <row r="9">
@@ -1618,88 +1618,88 @@
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>86.09</v>
+        <v>82.79024390243903</v>
       </c>
       <c r="J9" t="n">
-        <v>90.01000000000001</v>
+        <v>84.86</v>
       </c>
       <c r="K9" t="n">
-        <v>93.94</v>
+        <v>89.93000000000001</v>
       </c>
       <c r="L9" t="n">
-        <v>97.86</v>
+        <v>95.27</v>
       </c>
       <c r="M9" t="n">
-        <v>101.79</v>
+        <v>100.91</v>
       </c>
       <c r="N9" t="n">
-        <v>105.71</v>
+        <v>106.85</v>
       </c>
       <c r="O9" t="n">
-        <v>109.64</v>
+        <v>113.11</v>
       </c>
       <c r="P9" t="n">
-        <v>113.56</v>
+        <v>119.71</v>
       </c>
       <c r="Q9" t="n">
-        <v>117.49</v>
+        <v>126.67</v>
       </c>
       <c r="R9" t="n">
-        <v>121.41</v>
+        <v>133.99</v>
       </c>
       <c r="S9" t="n">
-        <v>125.34</v>
+        <v>141.71</v>
       </c>
       <c r="T9" t="n">
-        <v>129.27</v>
+        <v>149.84</v>
       </c>
       <c r="U9" t="n">
-        <v>133.19</v>
+        <v>158.41</v>
       </c>
       <c r="V9" t="n">
-        <v>137.12</v>
+        <v>167.78</v>
       </c>
       <c r="W9" t="n">
-        <v>141.04</v>
+        <v>177.58</v>
       </c>
       <c r="X9" t="n">
-        <v>144.97</v>
+        <v>187.83</v>
       </c>
       <c r="Y9" t="n">
-        <v>148.89</v>
+        <v>198.55</v>
       </c>
       <c r="Z9" t="n">
-        <v>152.82</v>
+        <v>209.76</v>
       </c>
       <c r="AA9" t="n">
-        <v>156.74</v>
+        <v>221.48</v>
       </c>
       <c r="AB9" t="n">
-        <v>160.67</v>
+        <v>233.73</v>
       </c>
       <c r="AC9" t="n">
-        <v>164.59</v>
+        <v>246.54</v>
       </c>
       <c r="AD9" t="n">
-        <v>168.52</v>
+        <v>259.91</v>
       </c>
       <c r="AE9" t="n">
-        <v>172.45</v>
+        <v>273.89</v>
       </c>
       <c r="AF9" t="n">
-        <v>176.37</v>
+        <v>288.49</v>
       </c>
       <c r="AG9" t="n">
-        <v>180.3</v>
+        <v>303.73</v>
       </c>
       <c r="AH9" t="n">
-        <v>184.22</v>
+        <v>319.65</v>
       </c>
       <c r="AI9" t="n">
-        <v>188.15</v>
+        <v>336.28</v>
       </c>
       <c r="AJ9" t="n">
-        <v>192.07</v>
+        <v>353.63</v>
       </c>
     </row>
     <row r="10">
@@ -1742,88 +1742,88 @@
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>129.58</v>
+        <v>115.9024390243902</v>
       </c>
       <c r="J10" t="n">
-        <v>134.09</v>
+        <v>118.8</v>
       </c>
       <c r="K10" t="n">
-        <v>138.6</v>
+        <v>123.85</v>
       </c>
       <c r="L10" t="n">
-        <v>143.11</v>
+        <v>129.07</v>
       </c>
       <c r="M10" t="n">
-        <v>147.62</v>
+        <v>134.47</v>
       </c>
       <c r="N10" t="n">
-        <v>152.12</v>
+        <v>140.06</v>
       </c>
       <c r="O10" t="n">
-        <v>156.63</v>
+        <v>145.85</v>
       </c>
       <c r="P10" t="n">
-        <v>161.14</v>
+        <v>151.84</v>
       </c>
       <c r="Q10" t="n">
-        <v>165.65</v>
+        <v>158.04</v>
       </c>
       <c r="R10" t="n">
-        <v>170.16</v>
+        <v>164.46</v>
       </c>
       <c r="S10" t="n">
-        <v>174.67</v>
+        <v>171.1</v>
       </c>
       <c r="T10" t="n">
-        <v>179.18</v>
+        <v>177.96</v>
       </c>
       <c r="U10" t="n">
-        <v>183.69</v>
+        <v>185.06</v>
       </c>
       <c r="V10" t="n">
-        <v>188.2</v>
+        <v>193.44</v>
       </c>
       <c r="W10" t="n">
-        <v>192.71</v>
+        <v>202.06</v>
       </c>
       <c r="X10" t="n">
-        <v>197.22</v>
+        <v>210.93</v>
       </c>
       <c r="Y10" t="n">
-        <v>201.73</v>
+        <v>220.06</v>
       </c>
       <c r="Z10" t="n">
-        <v>206.24</v>
+        <v>229.44</v>
       </c>
       <c r="AA10" t="n">
-        <v>210.75</v>
+        <v>239.09</v>
       </c>
       <c r="AB10" t="n">
-        <v>215.26</v>
+        <v>249.01</v>
       </c>
       <c r="AC10" t="n">
-        <v>219.76</v>
+        <v>259.21</v>
       </c>
       <c r="AD10" t="n">
-        <v>224.27</v>
+        <v>269.7</v>
       </c>
       <c r="AE10" t="n">
-        <v>228.78</v>
+        <v>280.48</v>
       </c>
       <c r="AF10" t="n">
-        <v>233.29</v>
+        <v>291.57</v>
       </c>
       <c r="AG10" t="n">
-        <v>237.8</v>
+        <v>302.96</v>
       </c>
       <c r="AH10" t="n">
-        <v>242.31</v>
+        <v>314.66</v>
       </c>
       <c r="AI10" t="n">
-        <v>246.82</v>
+        <v>326.69</v>
       </c>
       <c r="AJ10" t="n">
-        <v>251.33</v>
+        <v>339.06</v>
       </c>
     </row>
     <row r="11">
@@ -1866,88 +1866,88 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>47.17</v>
+        <v>57.95121951219512</v>
       </c>
       <c r="J11" t="n">
-        <v>48.61</v>
+        <v>59.4</v>
       </c>
       <c r="K11" t="n">
-        <v>50.06</v>
+        <v>62.77</v>
       </c>
       <c r="L11" t="n">
-        <v>51.5</v>
+        <v>66.31</v>
       </c>
       <c r="M11" t="n">
-        <v>52.94</v>
+        <v>70.03</v>
       </c>
       <c r="N11" t="n">
-        <v>54.39</v>
+        <v>73.94</v>
       </c>
       <c r="O11" t="n">
-        <v>55.83</v>
+        <v>78.05</v>
       </c>
       <c r="P11" t="n">
-        <v>57.27</v>
+        <v>82.36</v>
       </c>
       <c r="Q11" t="n">
-        <v>58.72</v>
+        <v>86.89</v>
       </c>
       <c r="R11" t="n">
-        <v>60.16</v>
+        <v>91.66</v>
       </c>
       <c r="S11" t="n">
-        <v>61.6</v>
+        <v>96.66</v>
       </c>
       <c r="T11" t="n">
-        <v>63.05</v>
+        <v>101.91</v>
       </c>
       <c r="U11" t="n">
-        <v>64.48999999999999</v>
+        <v>107.42</v>
       </c>
       <c r="V11" t="n">
-        <v>65.93000000000001</v>
+        <v>113.34</v>
       </c>
       <c r="W11" t="n">
-        <v>67.38</v>
+        <v>119.49</v>
       </c>
       <c r="X11" t="n">
-        <v>68.81999999999999</v>
+        <v>125.9</v>
       </c>
       <c r="Y11" t="n">
-        <v>70.27</v>
+        <v>132.57</v>
       </c>
       <c r="Z11" t="n">
-        <v>71.70999999999999</v>
+        <v>139.51</v>
       </c>
       <c r="AA11" t="n">
-        <v>73.15000000000001</v>
+        <v>146.74</v>
       </c>
       <c r="AB11" t="n">
-        <v>74.59999999999999</v>
+        <v>154.25</v>
       </c>
       <c r="AC11" t="n">
-        <v>76.04000000000001</v>
+        <v>162.07</v>
       </c>
       <c r="AD11" t="n">
-        <v>77.48</v>
+        <v>170.2</v>
       </c>
       <c r="AE11" t="n">
-        <v>78.93000000000001</v>
+        <v>178.66</v>
       </c>
       <c r="AF11" t="n">
-        <v>80.37</v>
+        <v>187.45</v>
       </c>
       <c r="AG11" t="n">
-        <v>81.81</v>
+        <v>196.59</v>
       </c>
       <c r="AH11" t="n">
-        <v>83.26000000000001</v>
+        <v>206.1</v>
       </c>
       <c r="AI11" t="n">
-        <v>84.7</v>
+        <v>215.97</v>
       </c>
       <c r="AJ11" t="n">
-        <v>86.14</v>
+        <v>226.23</v>
       </c>
     </row>
     <row r="12">
@@ -1990,88 +1990,88 @@
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>43.14</v>
+        <v>37.25853658536585</v>
       </c>
       <c r="J12" t="n">
-        <v>44.53</v>
+        <v>38.19</v>
       </c>
       <c r="K12" t="n">
-        <v>45.91</v>
+        <v>40.2</v>
       </c>
       <c r="L12" t="n">
-        <v>47.3</v>
+        <v>42.3</v>
       </c>
       <c r="M12" t="n">
-        <v>48.68</v>
+        <v>44.5</v>
       </c>
       <c r="N12" t="n">
-        <v>50.07</v>
+        <v>46.8</v>
       </c>
       <c r="O12" t="n">
-        <v>51.45</v>
+        <v>49.21</v>
       </c>
       <c r="P12" t="n">
-        <v>52.84</v>
+        <v>51.73</v>
       </c>
       <c r="Q12" t="n">
-        <v>54.22</v>
+        <v>54.37</v>
       </c>
       <c r="R12" t="n">
-        <v>55.61</v>
+        <v>57.13</v>
       </c>
       <c r="S12" t="n">
-        <v>56.99</v>
+        <v>60.02</v>
       </c>
       <c r="T12" t="n">
-        <v>58.37</v>
+        <v>63.03</v>
       </c>
       <c r="U12" t="n">
-        <v>59.76</v>
+        <v>66.19</v>
       </c>
       <c r="V12" t="n">
-        <v>61.14</v>
+        <v>69.68000000000001</v>
       </c>
       <c r="W12" t="n">
-        <v>62.53</v>
+        <v>73.31</v>
       </c>
       <c r="X12" t="n">
-        <v>63.91</v>
+        <v>77.08</v>
       </c>
       <c r="Y12" t="n">
-        <v>65.3</v>
+        <v>80.98999999999999</v>
       </c>
       <c r="Z12" t="n">
-        <v>66.68000000000001</v>
+        <v>85.04000000000001</v>
       </c>
       <c r="AA12" t="n">
-        <v>68.06999999999999</v>
+        <v>89.26000000000001</v>
       </c>
       <c r="AB12" t="n">
-        <v>69.45</v>
+        <v>93.63</v>
       </c>
       <c r="AC12" t="n">
-        <v>70.84</v>
+        <v>98.16</v>
       </c>
       <c r="AD12" t="n">
-        <v>72.22</v>
+        <v>102.87</v>
       </c>
       <c r="AE12" t="n">
-        <v>73.61</v>
+        <v>107.75</v>
       </c>
       <c r="AF12" t="n">
-        <v>74.98999999999999</v>
+        <v>112.81</v>
       </c>
       <c r="AG12" t="n">
-        <v>76.38</v>
+        <v>118.06</v>
       </c>
       <c r="AH12" t="n">
-        <v>77.76000000000001</v>
+        <v>123.5</v>
       </c>
       <c r="AI12" t="n">
-        <v>79.15000000000001</v>
+        <v>129.14</v>
       </c>
       <c r="AJ12" t="n">
-        <v>80.53</v>
+        <v>134.98</v>
       </c>
     </row>
     <row r="13">
@@ -2114,88 +2114,88 @@
         <v>0</v>
       </c>
       <c r="I13" t="n">
+        <v>1211.141463414634</v>
+      </c>
+      <c r="J13" t="n">
         <v>1241.42</v>
       </c>
-      <c r="J13" t="n">
-        <v>1278.67</v>
-      </c>
       <c r="K13" t="n">
-        <v>1315.91</v>
+        <v>1273.32</v>
       </c>
       <c r="L13" t="n">
-        <v>1353.15</v>
+        <v>1306.05</v>
       </c>
       <c r="M13" t="n">
-        <v>1390.4</v>
+        <v>1339.61</v>
       </c>
       <c r="N13" t="n">
-        <v>1427.64</v>
+        <v>1374.04</v>
       </c>
       <c r="O13" t="n">
-        <v>1464.88</v>
+        <v>1409.36</v>
       </c>
       <c r="P13" t="n">
-        <v>1502.12</v>
+        <v>1445.58</v>
       </c>
       <c r="Q13" t="n">
-        <v>1539.37</v>
+        <v>1482.73</v>
       </c>
       <c r="R13" t="n">
-        <v>1576.61</v>
+        <v>1520.83</v>
       </c>
       <c r="S13" t="n">
-        <v>1613.85</v>
+        <v>1559.92</v>
       </c>
       <c r="T13" t="n">
-        <v>1651.09</v>
+        <v>1600.01</v>
       </c>
       <c r="U13" t="n">
-        <v>1688.34</v>
+        <v>1641.13</v>
       </c>
       <c r="V13" t="n">
-        <v>1725.58</v>
+        <v>1667.55</v>
       </c>
       <c r="W13" t="n">
-        <v>1762.82</v>
+        <v>1694.4</v>
       </c>
       <c r="X13" t="n">
-        <v>1800.07</v>
+        <v>1721.68</v>
       </c>
       <c r="Y13" t="n">
-        <v>1837.31</v>
+        <v>1749.4</v>
       </c>
       <c r="Z13" t="n">
-        <v>1874.55</v>
+        <v>1777.56</v>
       </c>
       <c r="AA13" t="n">
-        <v>1911.79</v>
+        <v>1806.18</v>
       </c>
       <c r="AB13" t="n">
-        <v>1949.04</v>
+        <v>1835.26</v>
       </c>
       <c r="AC13" t="n">
-        <v>1986.28</v>
+        <v>1864.81</v>
       </c>
       <c r="AD13" t="n">
-        <v>2023.52</v>
+        <v>1894.83</v>
       </c>
       <c r="AE13" t="n">
-        <v>2060.76</v>
+        <v>1925.34</v>
       </c>
       <c r="AF13" t="n">
-        <v>2098.01</v>
+        <v>1956.34</v>
       </c>
       <c r="AG13" t="n">
-        <v>2135.25</v>
+        <v>1987.83</v>
       </c>
       <c r="AH13" t="n">
-        <v>2172.49</v>
+        <v>2019.84</v>
       </c>
       <c r="AI13" t="n">
-        <v>2209.74</v>
+        <v>2052.36</v>
       </c>
       <c r="AJ13" t="n">
-        <v>2246.98</v>
+        <v>2085.4</v>
       </c>
     </row>
     <row r="14">
@@ -2238,88 +2238,88 @@
         <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>20.33</v>
+        <v>20.69268292682927</v>
       </c>
       <c r="J14" t="n">
-        <v>21.26</v>
+        <v>21.21</v>
       </c>
       <c r="K14" t="n">
-        <v>22.19</v>
+        <v>22.25</v>
       </c>
       <c r="L14" t="n">
-        <v>23.12</v>
+        <v>23.33</v>
       </c>
       <c r="M14" t="n">
-        <v>24.04</v>
+        <v>24.46</v>
       </c>
       <c r="N14" t="n">
-        <v>24.97</v>
+        <v>25.63</v>
       </c>
       <c r="O14" t="n">
-        <v>25.9</v>
+        <v>26.86</v>
       </c>
       <c r="P14" t="n">
-        <v>26.83</v>
+        <v>28.13</v>
       </c>
       <c r="Q14" t="n">
-        <v>27.76</v>
+        <v>29.46</v>
       </c>
       <c r="R14" t="n">
-        <v>28.69</v>
+        <v>30.84</v>
       </c>
       <c r="S14" t="n">
-        <v>29.62</v>
+        <v>32.29</v>
       </c>
       <c r="T14" t="n">
-        <v>30.55</v>
+        <v>33.79</v>
       </c>
       <c r="U14" t="n">
-        <v>31.48</v>
+        <v>35.35</v>
       </c>
       <c r="V14" t="n">
-        <v>32.41</v>
+        <v>37.1</v>
       </c>
       <c r="W14" t="n">
-        <v>33.33</v>
+        <v>38.9</v>
       </c>
       <c r="X14" t="n">
-        <v>34.26</v>
+        <v>40.77</v>
       </c>
       <c r="Y14" t="n">
-        <v>35.19</v>
+        <v>42.7</v>
       </c>
       <c r="Z14" t="n">
-        <v>36.12</v>
+        <v>44.7</v>
       </c>
       <c r="AA14" t="n">
-        <v>37.05</v>
+        <v>46.76</v>
       </c>
       <c r="AB14" t="n">
-        <v>37.98</v>
+        <v>48.89</v>
       </c>
       <c r="AC14" t="n">
-        <v>38.91</v>
+        <v>51.09</v>
       </c>
       <c r="AD14" t="n">
-        <v>39.84</v>
+        <v>53.37</v>
       </c>
       <c r="AE14" t="n">
-        <v>40.77</v>
+        <v>55.72</v>
       </c>
       <c r="AF14" t="n">
-        <v>41.7</v>
+        <v>58.15</v>
       </c>
       <c r="AG14" t="n">
-        <v>42.62</v>
+        <v>60.66</v>
       </c>
       <c r="AH14" t="n">
-        <v>43.55</v>
+        <v>63.25</v>
       </c>
       <c r="AI14" t="n">
-        <v>44.48</v>
+        <v>65.93000000000001</v>
       </c>
       <c r="AJ14" t="n">
-        <v>45.41</v>
+        <v>68.69</v>
       </c>
     </row>
     <row r="15">
@@ -2362,88 +2362,88 @@
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>51.8</v>
+        <v>53.81463414634146</v>
       </c>
       <c r="J15" t="n">
-        <v>54.32</v>
+        <v>55.16</v>
       </c>
       <c r="K15" t="n">
-        <v>56.84</v>
+        <v>58.36</v>
       </c>
       <c r="L15" t="n">
-        <v>59.36</v>
+        <v>61.73</v>
       </c>
       <c r="M15" t="n">
-        <v>61.89</v>
+        <v>65.27</v>
       </c>
       <c r="N15" t="n">
-        <v>64.41</v>
+        <v>69</v>
       </c>
       <c r="O15" t="n">
-        <v>66.93000000000001</v>
+        <v>72.93000000000001</v>
       </c>
       <c r="P15" t="n">
-        <v>69.45999999999999</v>
+        <v>77.05</v>
       </c>
       <c r="Q15" t="n">
-        <v>71.98</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="R15" t="n">
-        <v>74.5</v>
+        <v>85.95999999999999</v>
       </c>
       <c r="S15" t="n">
-        <v>77.02</v>
+        <v>90.77</v>
       </c>
       <c r="T15" t="n">
-        <v>79.55</v>
+        <v>95.81999999999999</v>
       </c>
       <c r="U15" t="n">
-        <v>82.06999999999999</v>
+        <v>101.13</v>
       </c>
       <c r="V15" t="n">
-        <v>84.59</v>
+        <v>106.96</v>
       </c>
       <c r="W15" t="n">
-        <v>87.11</v>
+        <v>113.04</v>
       </c>
       <c r="X15" t="n">
-        <v>89.64</v>
+        <v>119.39</v>
       </c>
       <c r="Y15" t="n">
-        <v>92.16</v>
+        <v>126.03</v>
       </c>
       <c r="Z15" t="n">
-        <v>94.68000000000001</v>
+        <v>132.95</v>
       </c>
       <c r="AA15" t="n">
-        <v>97.2</v>
+        <v>140.17</v>
       </c>
       <c r="AB15" t="n">
-        <v>99.73</v>
+        <v>147.71</v>
       </c>
       <c r="AC15" t="n">
-        <v>102.25</v>
+        <v>155.57</v>
       </c>
       <c r="AD15" t="n">
-        <v>104.77</v>
+        <v>163.78</v>
       </c>
       <c r="AE15" t="n">
-        <v>107.29</v>
+        <v>172.33</v>
       </c>
       <c r="AF15" t="n">
-        <v>109.82</v>
+        <v>181.25</v>
       </c>
       <c r="AG15" t="n">
-        <v>112.34</v>
+        <v>190.56</v>
       </c>
       <c r="AH15" t="n">
-        <v>114.86</v>
+        <v>200.25</v>
       </c>
       <c r="AI15" t="n">
-        <v>117.38</v>
+        <v>210.36</v>
       </c>
       <c r="AJ15" t="n">
-        <v>119.91</v>
+        <v>220.89</v>
       </c>
     </row>
     <row r="16">
@@ -2486,88 +2486,88 @@
         <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>223.03</v>
+        <v>227.6682926829269</v>
       </c>
       <c r="J16" t="n">
-        <v>232.58</v>
+        <v>233.36</v>
       </c>
       <c r="K16" t="n">
-        <v>242.13</v>
+        <v>246.9</v>
       </c>
       <c r="L16" t="n">
-        <v>251.67</v>
+        <v>261.15</v>
       </c>
       <c r="M16" t="n">
-        <v>261.22</v>
+        <v>276.14</v>
       </c>
       <c r="N16" t="n">
-        <v>270.76</v>
+        <v>291.93</v>
       </c>
       <c r="O16" t="n">
-        <v>280.31</v>
+        <v>308.53</v>
       </c>
       <c r="P16" t="n">
-        <v>289.86</v>
+        <v>326</v>
       </c>
       <c r="Q16" t="n">
-        <v>299.4</v>
+        <v>344.37</v>
       </c>
       <c r="R16" t="n">
-        <v>308.95</v>
+        <v>363.7</v>
       </c>
       <c r="S16" t="n">
-        <v>318.49</v>
+        <v>384.02</v>
       </c>
       <c r="T16" t="n">
-        <v>328.04</v>
+        <v>405.39</v>
       </c>
       <c r="U16" t="n">
-        <v>337.59</v>
+        <v>427.87</v>
       </c>
       <c r="V16" t="n">
-        <v>347.13</v>
+        <v>452.51</v>
       </c>
       <c r="W16" t="n">
-        <v>356.68</v>
+        <v>478.25</v>
       </c>
       <c r="X16" t="n">
-        <v>366.22</v>
+        <v>505.13</v>
       </c>
       <c r="Y16" t="n">
-        <v>375.77</v>
+        <v>533.1799999999999</v>
       </c>
       <c r="Z16" t="n">
-        <v>385.31</v>
+        <v>562.47</v>
       </c>
       <c r="AA16" t="n">
-        <v>394.86</v>
+        <v>593.04</v>
       </c>
       <c r="AB16" t="n">
-        <v>404.41</v>
+        <v>624.9299999999999</v>
       </c>
       <c r="AC16" t="n">
-        <v>413.95</v>
+        <v>658.2</v>
       </c>
       <c r="AD16" t="n">
-        <v>423.5</v>
+        <v>692.91</v>
       </c>
       <c r="AE16" t="n">
-        <v>433.04</v>
+        <v>729.1</v>
       </c>
       <c r="AF16" t="n">
-        <v>442.59</v>
+        <v>766.85</v>
       </c>
       <c r="AG16" t="n">
-        <v>452.14</v>
+        <v>806.2</v>
       </c>
       <c r="AH16" t="n">
-        <v>461.68</v>
+        <v>847.22</v>
       </c>
       <c r="AI16" t="n">
-        <v>471.23</v>
+        <v>889.98</v>
       </c>
       <c r="AJ16" t="n">
-        <v>480.77</v>
+        <v>934.54</v>
       </c>
     </row>
     <row r="17">
@@ -2610,88 +2610,88 @@
         <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>81.55</v>
+        <v>66.23414634146341</v>
       </c>
       <c r="J17" t="n">
-        <v>86.75</v>
+        <v>67.89</v>
       </c>
       <c r="K17" t="n">
-        <v>91.95</v>
+        <v>71.53</v>
       </c>
       <c r="L17" t="n">
-        <v>97.15000000000001</v>
+        <v>75.34</v>
       </c>
       <c r="M17" t="n">
-        <v>102.36</v>
+        <v>79.34</v>
       </c>
       <c r="N17" t="n">
-        <v>107.56</v>
+        <v>83.53</v>
       </c>
       <c r="O17" t="n">
-        <v>112.76</v>
+        <v>87.91</v>
       </c>
       <c r="P17" t="n">
-        <v>117.97</v>
+        <v>92.51000000000001</v>
       </c>
       <c r="Q17" t="n">
-        <v>123.17</v>
+        <v>97.31999999999999</v>
       </c>
       <c r="R17" t="n">
-        <v>128.37</v>
+        <v>102.35</v>
       </c>
       <c r="S17" t="n">
-        <v>133.57</v>
+        <v>107.63</v>
       </c>
       <c r="T17" t="n">
-        <v>138.78</v>
+        <v>113.15</v>
       </c>
       <c r="U17" t="n">
-        <v>143.98</v>
+        <v>118.93</v>
       </c>
       <c r="V17" t="n">
-        <v>149.18</v>
+        <v>125.51</v>
       </c>
       <c r="W17" t="n">
-        <v>154.38</v>
+        <v>132.36</v>
       </c>
       <c r="X17" t="n">
-        <v>159.59</v>
+        <v>139.5</v>
       </c>
       <c r="Y17" t="n">
-        <v>164.79</v>
+        <v>146.94</v>
       </c>
       <c r="Z17" t="n">
-        <v>169.99</v>
+        <v>154.68</v>
       </c>
       <c r="AA17" t="n">
-        <v>175.2</v>
+        <v>162.73</v>
       </c>
       <c r="AB17" t="n">
-        <v>180.4</v>
+        <v>171.12</v>
       </c>
       <c r="AC17" t="n">
-        <v>185.6</v>
+        <v>179.85</v>
       </c>
       <c r="AD17" t="n">
-        <v>190.8</v>
+        <v>188.92</v>
       </c>
       <c r="AE17" t="n">
-        <v>196.01</v>
+        <v>198.37</v>
       </c>
       <c r="AF17" t="n">
-        <v>201.21</v>
+        <v>208.19</v>
       </c>
       <c r="AG17" t="n">
-        <v>206.41</v>
+        <v>218.41</v>
       </c>
       <c r="AH17" t="n">
-        <v>211.61</v>
+        <v>229.03</v>
       </c>
       <c r="AI17" t="n">
-        <v>216.82</v>
+        <v>240.08</v>
       </c>
       <c r="AJ17" t="n">
-        <v>222.02</v>
+        <v>251.56</v>
       </c>
     </row>
     <row r="18">
@@ -2734,88 +2734,88 @@
         <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>27.94</v>
+        <v>28.97560975609756</v>
       </c>
       <c r="J18" t="n">
-        <v>28.58</v>
+        <v>29.7</v>
       </c>
       <c r="K18" t="n">
-        <v>29.23</v>
+        <v>31.04</v>
       </c>
       <c r="L18" t="n">
-        <v>29.87</v>
+        <v>32.42</v>
       </c>
       <c r="M18" t="n">
-        <v>30.52</v>
+        <v>33.86</v>
       </c>
       <c r="N18" t="n">
-        <v>31.16</v>
+        <v>35.36</v>
       </c>
       <c r="O18" t="n">
-        <v>31.81</v>
+        <v>36.91</v>
       </c>
       <c r="P18" t="n">
-        <v>32.45</v>
+        <v>38.52</v>
       </c>
       <c r="Q18" t="n">
-        <v>33.1</v>
+        <v>40.19</v>
       </c>
       <c r="R18" t="n">
-        <v>33.75</v>
+        <v>41.92</v>
       </c>
       <c r="S18" t="n">
-        <v>34.39</v>
+        <v>43.72</v>
       </c>
       <c r="T18" t="n">
-        <v>35.04</v>
+        <v>45.59</v>
       </c>
       <c r="U18" t="n">
-        <v>35.68</v>
+        <v>47.52</v>
       </c>
       <c r="V18" t="n">
-        <v>36.33</v>
+        <v>49.72</v>
       </c>
       <c r="W18" t="n">
-        <v>36.97</v>
+        <v>51.99</v>
       </c>
       <c r="X18" t="n">
-        <v>37.62</v>
+        <v>54.33</v>
       </c>
       <c r="Y18" t="n">
-        <v>38.26</v>
+        <v>56.73</v>
       </c>
       <c r="Z18" t="n">
-        <v>38.91</v>
+        <v>59.21</v>
       </c>
       <c r="AA18" t="n">
-        <v>39.55</v>
+        <v>61.76</v>
       </c>
       <c r="AB18" t="n">
-        <v>40.2</v>
+        <v>64.38</v>
       </c>
       <c r="AC18" t="n">
-        <v>40.84</v>
+        <v>67.09</v>
       </c>
       <c r="AD18" t="n">
-        <v>41.49</v>
+        <v>69.87</v>
       </c>
       <c r="AE18" t="n">
-        <v>42.14</v>
+        <v>72.73999999999999</v>
       </c>
       <c r="AF18" t="n">
-        <v>42.78</v>
+        <v>75.68000000000001</v>
       </c>
       <c r="AG18" t="n">
-        <v>43.43</v>
+        <v>78.72</v>
       </c>
       <c r="AH18" t="n">
-        <v>44.07</v>
+        <v>81.84</v>
       </c>
       <c r="AI18" t="n">
-        <v>44.72</v>
+        <v>85.05</v>
       </c>
       <c r="AJ18" t="n">
-        <v>45.36</v>
+        <v>88.36</v>
       </c>
     </row>
     <row r="19">
@@ -2858,88 +2858,88 @@
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>50.51</v>
+        <v>49.67804878048781</v>
       </c>
       <c r="J19" t="n">
-        <v>51.7</v>
+        <v>50.92</v>
       </c>
       <c r="K19" t="n">
-        <v>52.89</v>
+        <v>52.61</v>
       </c>
       <c r="L19" t="n">
-        <v>54.09</v>
+        <v>54.35</v>
       </c>
       <c r="M19" t="n">
-        <v>55.28</v>
+        <v>56.13</v>
       </c>
       <c r="N19" t="n">
-        <v>56.47</v>
+        <v>57.95</v>
       </c>
       <c r="O19" t="n">
-        <v>57.66</v>
+        <v>59.81</v>
       </c>
       <c r="P19" t="n">
-        <v>58.85</v>
+        <v>61.72</v>
       </c>
       <c r="Q19" t="n">
-        <v>60.05</v>
+        <v>63.68</v>
       </c>
       <c r="R19" t="n">
-        <v>61.24</v>
+        <v>65.68000000000001</v>
       </c>
       <c r="S19" t="n">
-        <v>62.43</v>
+        <v>67.73</v>
       </c>
       <c r="T19" t="n">
-        <v>63.62</v>
+        <v>69.83</v>
       </c>
       <c r="U19" t="n">
-        <v>64.81999999999999</v>
+        <v>71.98</v>
       </c>
       <c r="V19" t="n">
-        <v>66.01000000000001</v>
+        <v>74.69</v>
       </c>
       <c r="W19" t="n">
-        <v>67.2</v>
+        <v>77.44</v>
       </c>
       <c r="X19" t="n">
-        <v>68.39</v>
+        <v>80.23999999999999</v>
       </c>
       <c r="Y19" t="n">
-        <v>69.58</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="Z19" t="n">
-        <v>70.78</v>
+        <v>86</v>
       </c>
       <c r="AA19" t="n">
-        <v>71.97</v>
+        <v>88.95999999999999</v>
       </c>
       <c r="AB19" t="n">
-        <v>73.16</v>
+        <v>91.97</v>
       </c>
       <c r="AC19" t="n">
-        <v>74.34999999999999</v>
+        <v>95.03</v>
       </c>
       <c r="AD19" t="n">
-        <v>75.54000000000001</v>
+        <v>98.15000000000001</v>
       </c>
       <c r="AE19" t="n">
-        <v>76.73999999999999</v>
+        <v>101.32</v>
       </c>
       <c r="AF19" t="n">
-        <v>77.93000000000001</v>
+        <v>104.54</v>
       </c>
       <c r="AG19" t="n">
-        <v>79.12</v>
+        <v>107.83</v>
       </c>
       <c r="AH19" t="n">
-        <v>80.31</v>
+        <v>111.17</v>
       </c>
       <c r="AI19" t="n">
-        <v>81.5</v>
+        <v>114.57</v>
       </c>
       <c r="AJ19" t="n">
-        <v>82.7</v>
+        <v>118.03</v>
       </c>
     </row>
     <row r="20">
@@ -2982,88 +2982,88 @@
         <v>0</v>
       </c>
       <c r="I20" t="n">
-        <v>3.13</v>
+        <v>6.204878048780489</v>
       </c>
       <c r="J20" t="n">
-        <v>3.33</v>
+        <v>6.36</v>
       </c>
       <c r="K20" t="n">
-        <v>3.53</v>
+        <v>6.67</v>
       </c>
       <c r="L20" t="n">
-        <v>3.73</v>
+        <v>6.98</v>
       </c>
       <c r="M20" t="n">
-        <v>3.92</v>
+        <v>7.31</v>
       </c>
       <c r="N20" t="n">
-        <v>4.12</v>
+        <v>7.65</v>
       </c>
       <c r="O20" t="n">
-        <v>4.32</v>
+        <v>8.01</v>
       </c>
       <c r="P20" t="n">
-        <v>4.52</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="Q20" t="n">
-        <v>4.72</v>
+        <v>8.76</v>
       </c>
       <c r="R20" t="n">
-        <v>4.92</v>
+        <v>9.16</v>
       </c>
       <c r="S20" t="n">
-        <v>5.12</v>
+        <v>9.58</v>
       </c>
       <c r="T20" t="n">
-        <v>5.32</v>
+        <v>10.01</v>
       </c>
       <c r="U20" t="n">
-        <v>5.52</v>
+        <v>10.46</v>
       </c>
       <c r="V20" t="n">
-        <v>5.72</v>
+        <v>10.95</v>
       </c>
       <c r="W20" t="n">
-        <v>5.92</v>
+        <v>11.45</v>
       </c>
       <c r="X20" t="n">
-        <v>6.12</v>
+        <v>11.97</v>
       </c>
       <c r="Y20" t="n">
-        <v>6.32</v>
+        <v>12.51</v>
       </c>
       <c r="Z20" t="n">
-        <v>6.52</v>
+        <v>13.06</v>
       </c>
       <c r="AA20" t="n">
-        <v>6.72</v>
+        <v>13.63</v>
       </c>
       <c r="AB20" t="n">
-        <v>6.92</v>
+        <v>14.22</v>
       </c>
       <c r="AC20" t="n">
-        <v>7.12</v>
+        <v>14.82</v>
       </c>
       <c r="AD20" t="n">
-        <v>7.32</v>
+        <v>15.45</v>
       </c>
       <c r="AE20" t="n">
-        <v>7.52</v>
+        <v>16.09</v>
       </c>
       <c r="AF20" t="n">
-        <v>7.72</v>
+        <v>16.75</v>
       </c>
       <c r="AG20" t="n">
-        <v>7.91</v>
+        <v>17.43</v>
       </c>
       <c r="AH20" t="n">
-        <v>8.109999999999999</v>
+        <v>18.13</v>
       </c>
       <c r="AI20" t="n">
-        <v>8.31</v>
+        <v>18.85</v>
       </c>
       <c r="AJ20" t="n">
-        <v>8.51</v>
+        <v>19.59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>